<commit_message>
chore: fix tracker Phase 6 — clear orphaned W3-W8 labels from merged spacer rows
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -14436,11 +14436,7 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="53" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
-      </c>
+      <c r="A23" s="53" t="n"/>
       <c r="B23" s="103" t="n"/>
       <c r="C23" s="103" t="n"/>
       <c r="D23" s="103" t="n"/>
@@ -14633,11 +14629,7 @@
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="48" t="inlineStr">
-        <is>
-          <t>W4</t>
-        </is>
-      </c>
+      <c r="A28" s="48" t="n"/>
       <c r="B28" s="103" t="n"/>
       <c r="C28" s="103" t="n"/>
       <c r="D28" s="103" t="n"/>
@@ -14830,11 +14822,7 @@
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="48" t="inlineStr">
-        <is>
-          <t>W5</t>
-        </is>
-      </c>
+      <c r="A33" s="48" t="n"/>
       <c r="B33" s="103" t="n"/>
       <c r="C33" s="103" t="n"/>
       <c r="D33" s="103" t="n"/>
@@ -15027,11 +15015,7 @@
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="48" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
+      <c r="A38" s="48" t="n"/>
       <c r="B38" s="103" t="n"/>
       <c r="C38" s="103" t="n"/>
       <c r="D38" s="103" t="n"/>
@@ -15148,11 +15132,7 @@
       <c r="P41" s="104" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="65" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
+      <c r="A42" s="65" t="n"/>
       <c r="B42" s="103" t="n"/>
       <c r="C42" s="103" t="n"/>
       <c r="D42" s="103" t="n"/>
@@ -15573,11 +15553,7 @@
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="43" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
+      <c r="A50" s="43" t="n"/>
       <c r="B50" s="103" t="n"/>
       <c r="C50" s="103" t="n"/>
       <c r="D50" s="103" t="n"/>
@@ -15770,11 +15746,7 @@
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="48" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
+      <c r="A55" s="48" t="n"/>
       <c r="B55" s="103" t="n"/>
       <c r="C55" s="103" t="n"/>
       <c r="D55" s="103" t="n"/>

</xml_diff>

<commit_message>
tracker: reorder frontend tasks to sequential F01-F06 order
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -15437,12 +15437,12 @@
       </c>
       <c r="B46" s="89" t="inlineStr">
         <is>
-          <t>P6-F04</t>
+          <t>P6-F01</t>
         </is>
       </c>
       <c r="C46" s="18" t="inlineStr">
         <is>
-          <t>feature/swiggy-frontend-connectors</t>
+          <t>feature/swiggy-frontend-market</t>
         </is>
       </c>
       <c r="D46" s="18" t="inlineStr">
@@ -15452,17 +15452,17 @@
       </c>
       <c r="E46" s="18" t="inlineStr">
         <is>
-          <t>/connectors page — data source management</t>
+          <t>Market intelligence panel (planning results page)</t>
         </is>
       </c>
       <c r="F46" s="18" t="inlineStr">
         <is>
-          <t>New route /connectors. Lists connectors with status badges (Connected/Disconnected/Error). Shows last sync time, records synced, data freshness. Connect button triggers OAuth flow. Disconnect revokes token. Error state shows last error + reconnect. Works for Swiggy + future POS connector.</t>
+          <t>New panel on /runs/{id}. Competitor pricing table: your price vs area avg vs cheapest competitor per dish category. Area occupancy badge (HIGH/MEDIUM/LOW). Instamart prices for shortage items. Pricing alerts (red if &gt;20% above area avg). Hidden when market_intel_output absent.</t>
         </is>
       </c>
       <c r="G46" s="18" t="inlineStr">
         <is>
-          <t>feat: /connectors page — platform data source management with OAuth connect flow</t>
+          <t>feat: market intelligence panel — competitor pricing + area occupancy on planning results</t>
         </is>
       </c>
       <c r="H46" s="18" t="inlineStr">
@@ -15477,7 +15477,7 @@
       </c>
       <c r="J46" s="25" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K46" s="89" t="inlineStr">
@@ -15496,12 +15496,12 @@
       </c>
       <c r="O46" s="18" t="inlineStr">
         <is>
-          <t>P6-S01</t>
+          <t>P6-S10</t>
         </is>
       </c>
       <c r="P46" s="18" t="inlineStr">
         <is>
-          <t>Can build now — reads from connectors table (already exists via P6-S02)</t>
+          <t>Depends on P6-S11 (market_intel_output in plan API response)</t>
         </is>
       </c>
     </row>
@@ -15513,12 +15513,12 @@
       </c>
       <c r="B47" s="86" t="inlineStr">
         <is>
-          <t>P6-F06</t>
+          <t>P6-F02</t>
         </is>
       </c>
       <c r="C47" s="23" t="inlineStr">
         <is>
-          <t>feature/swiggy-frontend-market</t>
+          <t>feature/swiggy-frontend-actions</t>
         </is>
       </c>
       <c r="D47" s="23" t="inlineStr">
@@ -15528,17 +15528,17 @@
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
-          <t>Dashboard enhancements</t>
+          <t>Action queue UI + procurement tracker</t>
         </is>
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t>Add to existing dashboard: connector status widget (data source health bar), brief mode trigger button, today's Swiggy KPIs (orders today, delivery rating, top Swiggy seller), data_sources column on /runs list.</t>
+          <t>New section below plan output. Lists pending actions with type badge. Approve/Reject buttons for APPROVE_REQUIRED. Instamart cart preview modal (items, total, ETA) before approving checkout. Procurement tracker in inventory panel: placed orders, status, ETA.</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
         <is>
-          <t>feat: dashboard — connector status widget, brief trigger, live Swiggy KPIs, data_sources on runs list</t>
+          <t>feat: action queue UI — approve/reject with cart preview, procurement tracker</t>
         </is>
       </c>
       <c r="H47" s="23" t="inlineStr">
@@ -15553,7 +15553,7 @@
       </c>
       <c r="J47" s="25" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K47" s="86" t="inlineStr">
@@ -15572,12 +15572,12 @@
       </c>
       <c r="O47" s="23" t="inlineStr">
         <is>
-          <t>P6-S01</t>
+          <t>P6-S13</t>
         </is>
       </c>
       <c r="P47" s="23" t="inlineStr">
         <is>
-          <t>Can build now — connector status widget reads connectors table</t>
+          <t>Depends on P6-S14 (action_queue in plan API response)</t>
         </is>
       </c>
     </row>
@@ -15589,12 +15589,12 @@
       </c>
       <c r="B48" s="89" t="inlineStr">
         <is>
-          <t>P6-F01</t>
+          <t>P6-F03</t>
         </is>
       </c>
       <c r="C48" s="18" t="inlineStr">
         <is>
-          <t>feature/swiggy-frontend-market</t>
+          <t>feature/swiggy-frontend-brief</t>
         </is>
       </c>
       <c r="D48" s="18" t="inlineStr">
@@ -15604,17 +15604,17 @@
       </c>
       <c r="E48" s="18" t="inlineStr">
         <is>
-          <t>Market intelligence panel (planning results page)</t>
+          <t>/brief page — daily morning briefing</t>
         </is>
       </c>
       <c r="F48" s="18" t="inlineStr">
         <is>
-          <t>New panel on /runs/{id}. Competitor pricing table: your price vs area avg vs cheapest competitor per dish category. Area occupancy badge (HIGH/MEDIUM/LOW). Instamart prices for shortage items. Pricing alerts (red if &gt;20% above area avg). Hidden when market_intel_output absent.</t>
+          <t>New route /brief. Overnight Swiggy performance (orders, avg delivery time, late %), today's demand forecast vs yesterday, top 3 action priorities, market snapshot. Auto-refreshes if brief is stale. Empty state when no brief yet.</t>
         </is>
       </c>
       <c r="G48" s="18" t="inlineStr">
         <is>
-          <t>feat: market intelligence panel — competitor pricing + area occupancy on planning results</t>
+          <t>feat: /brief page — daily morning operational briefing</t>
         </is>
       </c>
       <c r="H48" s="18" t="inlineStr">
@@ -15629,7 +15629,7 @@
       </c>
       <c r="J48" s="30" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K48" s="89" t="inlineStr">
@@ -15648,12 +15648,12 @@
       </c>
       <c r="O48" s="18" t="inlineStr">
         <is>
-          <t>P6-S10</t>
+          <t>P6-S16</t>
         </is>
       </c>
       <c r="P48" s="18" t="inlineStr">
         <is>
-          <t>Depends on P6-S11 (market_intel_output in plan API response)</t>
+          <t>Depends on P6-S17 (BriefingService)</t>
         </is>
       </c>
     </row>
@@ -15665,12 +15665,12 @@
       </c>
       <c r="B49" s="86" t="inlineStr">
         <is>
-          <t>P6-F02</t>
+          <t>P6-F04</t>
         </is>
       </c>
       <c r="C49" s="23" t="inlineStr">
         <is>
-          <t>feature/swiggy-frontend-actions</t>
+          <t>feature/swiggy-frontend-connectors</t>
         </is>
       </c>
       <c r="D49" s="23" t="inlineStr">
@@ -15680,17 +15680,17 @@
       </c>
       <c r="E49" s="23" t="inlineStr">
         <is>
-          <t>Action queue UI + procurement tracker</t>
+          <t>/connectors page — data source management</t>
         </is>
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
-          <t>New section below plan output. Lists pending actions with type badge. Approve/Reject buttons for APPROVE_REQUIRED. Instamart cart preview modal (items, total, ETA) before approving checkout. Procurement tracker in inventory panel: placed orders, status, ETA.</t>
+          <t>New route /connectors. Lists connectors with status badges (Connected/Disconnected/Error). Shows last sync time, records synced, data freshness. Connect button triggers OAuth flow. Disconnect revokes token. Error state shows last error + reconnect. Works for Swiggy + future POS connector.</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
         <is>
-          <t>feat: action queue UI — approve/reject with cart preview, procurement tracker</t>
+          <t>feat: /connectors page — platform data source management with OAuth connect flow</t>
         </is>
       </c>
       <c r="H49" s="23" t="inlineStr">
@@ -15705,7 +15705,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="K49" s="86" t="inlineStr">
@@ -15724,12 +15724,12 @@
       </c>
       <c r="O49" s="23" t="inlineStr">
         <is>
-          <t>P6-S13</t>
+          <t>P6-S01</t>
         </is>
       </c>
       <c r="P49" s="23" t="inlineStr">
         <is>
-          <t>Depends on P6-S14 (action_queue in plan API response)</t>
+          <t>Can build now — reads from connectors table (already exists via P6-S02)</t>
         </is>
       </c>
     </row>
@@ -15741,12 +15741,12 @@
       </c>
       <c r="B50" s="88" t="inlineStr">
         <is>
-          <t>P6-F03</t>
+          <t>P6-F05</t>
         </is>
       </c>
       <c r="C50" s="28" t="inlineStr">
         <is>
-          <t>feature/swiggy-frontend-brief</t>
+          <t>feature/swiggy-frontend-live</t>
         </is>
       </c>
       <c r="D50" s="28" t="inlineStr">
@@ -15756,17 +15756,17 @@
       </c>
       <c r="E50" s="28" t="inlineStr">
         <is>
-          <t>/brief page — daily morning briefing</t>
+          <t>/live page — real-time service monitor</t>
         </is>
       </c>
       <c r="F50" s="28" t="inlineStr">
         <is>
-          <t>New route /brief. Overnight Swiggy performance (orders, avg delivery time, late %), today's demand forecast vs yesterday, top 3 action priorities, market snapshot. Auto-refreshes if brief is stale. Empty state when no brief yet.</t>
+          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S18). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
         </is>
       </c>
       <c r="G50" s="28" t="inlineStr">
         <is>
-          <t>feat: /brief page — daily morning operational briefing</t>
+          <t>feat: /live page — SSE kitchen display for active orders and procurement tracking</t>
         </is>
       </c>
       <c r="H50" s="28" t="inlineStr">
@@ -15800,12 +15800,12 @@
       </c>
       <c r="O50" s="28" t="inlineStr">
         <is>
-          <t>P6-S16</t>
+          <t>P6-S18</t>
         </is>
       </c>
       <c r="P50" s="28" t="inlineStr">
         <is>
-          <t>Depends on P6-S17 (BriefingService)</t>
+          <t>SSE events render in real time; ETA countdown ticks; alert banner fires on delivery spike; Swiggy branding visible; inactive state shown outside service hours.</t>
         </is>
       </c>
     </row>
@@ -15817,12 +15817,12 @@
       </c>
       <c r="B51" s="86" t="inlineStr">
         <is>
-          <t>P6-F05</t>
+          <t>P6-F06</t>
         </is>
       </c>
       <c r="C51" s="23" t="inlineStr">
         <is>
-          <t>feature/swiggy-frontend-live</t>
+          <t>feature/swiggy-frontend-market</t>
         </is>
       </c>
       <c r="D51" s="23" t="inlineStr">
@@ -15832,17 +15832,17 @@
       </c>
       <c r="E51" s="23" t="inlineStr">
         <is>
-          <t>/live page — real-time service monitor</t>
+          <t>Dashboard enhancements</t>
         </is>
       </c>
       <c r="F51" s="23" t="inlineStr">
         <is>
-          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S18). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
+          <t>Add to existing dashboard: connector status widget (data source health bar), brief mode trigger button, today's Swiggy KPIs (orders today, delivery rating, top Swiggy seller), data_sources column on /runs list.</t>
         </is>
       </c>
       <c r="G51" s="23" t="inlineStr">
         <is>
-          <t>feat: /live page — SSE kitchen display for active orders and procurement tracking</t>
+          <t>feat: dashboard — connector status widget, brief trigger, live Swiggy KPIs, data_sources on runs list</t>
         </is>
       </c>
       <c r="H51" s="23" t="inlineStr">
@@ -15876,12 +15876,12 @@
       </c>
       <c r="O51" s="23" t="inlineStr">
         <is>
-          <t>P6-S18</t>
+          <t>P6-S01</t>
         </is>
       </c>
       <c r="P51" s="23" t="inlineStr">
         <is>
-          <t>SSE events render in real time; ETA countdown ticks; alert banner fires on delivery spike; Swiggy branding visible; inactive state shown outside service hours.</t>
+          <t>Can build now — connector status widget reads connectors table</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: mark P6-S07 In Progress — start 2026-06-30
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -288,7 +289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -557,6 +558,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -14200,7 +14204,7 @@
       </c>
       <c r="I21" s="19" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J21" s="25" t="inlineStr">
@@ -14213,7 +14217,9 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L21" s="88" t="n"/>
+      <c r="L21" s="98" t="n">
+        <v>46203</v>
+      </c>
       <c r="M21" s="88" t="inlineStr">
         <is>
           <t>W3</t>

</xml_diff>

<commit_message>
tracker: mark P6-S07/S08/S09 Completed — all 3 enrichers done 2026-06-30
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -289,7 +289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -561,6 +561,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -14204,7 +14207,7 @@
       </c>
       <c r="I21" s="19" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J21" s="25" t="inlineStr">
@@ -14220,13 +14223,11 @@
       <c r="L21" s="98" t="n">
         <v>46203</v>
       </c>
-      <c r="M21" s="88" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
+      <c r="M21" s="98" t="n">
+        <v>46203</v>
       </c>
       <c r="N21" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O21" s="28" t="inlineStr">
         <is>
@@ -14282,7 +14283,7 @@
       </c>
       <c r="I22" s="19" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J22" s="25" t="inlineStr">
@@ -14296,13 +14297,11 @@
         </is>
       </c>
       <c r="L22" s="86" t="n"/>
-      <c r="M22" s="86" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
+      <c r="M22" s="99" t="n">
+        <v>46203</v>
       </c>
       <c r="N22" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" s="23" t="inlineStr">
         <is>
@@ -14358,7 +14357,7 @@
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J23" s="25" t="inlineStr">
@@ -14372,13 +14371,11 @@
         </is>
       </c>
       <c r="L23" s="88" t="n"/>
-      <c r="M23" s="88" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
+      <c r="M23" s="98" t="n">
+        <v>46203</v>
       </c>
       <c r="N23" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(P6-S11): market_intel_node — 10th parallel LangGraph node, Swiggy-powered market awareness
- New market_intel_node runs CompetitorEnricher + OccupancyEnricher +
  ProcurementEnricher concurrently via MarketIntelService
- Wired into parallel fan-out: qdrant_enrichment → market_intel → menu_intelligence
  alongside reservation / complaint_intelligence / inventory
- graph.py: MARKET_INTEL constant, node registered with swiggy_client dep,
  fan-out + fan-in edges, SSE map entry, start hint, completion hint
- aggregator: market_intel_output included in bundle + critic summary section
  ([Market Intel — Swiggy] area occupancy / pricing alerts / procurement options)
- SwiggyMCPClient instantiated once in build_graph, injectable via deps
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -296,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -553,6 +553,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -14519,7 +14522,7 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J27" s="25" t="inlineStr">
@@ -14532,14 +14535,14 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L27" s="27" t="n"/>
-      <c r="M27" s="27" t="inlineStr">
-        <is>
-          <t>W4</t>
-        </is>
+      <c r="L27" s="94" t="n">
+        <v>46204</v>
+      </c>
+      <c r="M27" s="94" t="n">
+        <v>46204</v>
       </c>
       <c r="N27" s="29" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O27" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(P6-S12): dineout_manager_node — own Dineout slot monitoring wired into planning pipeline
- New dineout_manager_node (11th parallel node) checks YOUR restaurant's
  Dineout slot availability for tonight via get_available_slots
- Flags open_more_recommended when >50% of dinner slots have low availability
- Wired into fan-out: qdrant_enrichment → dineout_manager → menu_intelligence
  (alongside reservation / complaint / inventory / market_intel)
- graph.py: DINEOUT_MANAGER constant, node registered with swiggy_client dep,
  fan-out + fan-in edges, SSE map, start hint, completion hint
- aggregator: dineout_manager_output in bundle + critic summary section
- settings.py: SWIGGY_DINEOUT_RESTAURANT_ID optional field added
- Degrades gracefully — no-op if ID not configured or Swiggy unavailable
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -14598,7 +14598,7 @@
       </c>
       <c r="I28" s="19" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J28" s="25" t="inlineStr">
@@ -14611,14 +14611,14 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L28" s="27" t="n"/>
-      <c r="M28" s="27" t="inlineStr">
-        <is>
-          <t>W4</t>
-        </is>
+      <c r="L28" s="94" t="n">
+        <v>46204</v>
+      </c>
+      <c r="M28" s="94" t="n">
+        <v>46204</v>
       </c>
       <c r="N28" s="29" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O28" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(P6-S13): assumption diffs 5+6 — market pricing vs menu, dineout slots vs reservation occupancy
Diff 5 (market_intel vs menu_intelligence):
  market_intel found N Swiggy pricing alerts (our items above area avg) but
  menu_intel is planning to push those same items — flags competitiveness risk
  before volume is driven on overpriced dishes

Diff 6 (dineout_manager vs reservation):
  dineout_manager found own Dineout slots nearly full AND reservation predicts
  >80% internal occupancy — compound demand signal triggers full-house staffing
  warning and open-more-slots recommendation

Also: aggregator assumptions bundle now includes dineout_manager_assumptions
alongside the existing 5 node assumptions, enabling diff 6 to read them.
Total active assumption diffs: 5 (Diff 1 removed, 2-6 active)
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -14674,7 +14674,7 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J29" s="30" t="inlineStr">
@@ -14687,14 +14687,14 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L29" s="27" t="n"/>
-      <c r="M29" s="27" t="inlineStr">
-        <is>
-          <t>W4</t>
-        </is>
+      <c r="L29" s="94" t="n">
+        <v>46204</v>
+      </c>
+      <c r="M29" s="94" t="n">
+        <v>46204</v>
       </c>
       <c r="N29" s="29" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O29" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
tracker: rebuild Phase 6+ in sequential execution order — add P7-S01/S02/S03/S04/S05/S07, demo checkpoint marked
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -13093,7 +13093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P63"/>
+  <dimension ref="A1:P64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.109375" customWidth="1" style="81" min="1" max="1"/>
@@ -14708,1827 +14708,2149 @@
       </c>
     </row>
     <row r="30" ht="52.05" customHeight="1" s="81">
-      <c r="A30" s="27" t="inlineStr">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DEMO SPRINT — Record end-to-end demo after P7-S04</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="52.05" customHeight="1" s="81">
+      <c r="A31" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="B30" s="27" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>P6-S13c</t>
         </is>
       </c>
-      <c r="C30" s="28" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>feature/swiggy-chatbot-tools</t>
         </is>
       </c>
-      <c r="D30" s="28" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="E30" s="28" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Swiggy-aware chatbot tools — HIGH PRIORITY FOR DEMO</t>
         </is>
       </c>
-      <c r="F30" s="28" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Add 3 Groq function-calling tools to the existing agentic chatbot (P6-S04). search_menu(query, addressId): answers questions like 'what is the avg biryani price near me?' get_food_orders(addressId): answers 'what were my top Swiggy items last week?' search_products(query, addressId): answers 'what does cream cost on Instamart right now?' Makes the chatbot genuinely Swiggy-aware — very demo-friendly for the Swiggy team.</t>
         </is>
       </c>
-      <c r="G30" s="28" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>feat: Swiggy chatbot tools — search_menu, get_food_orders, search_products via Groq function calling</t>
         </is>
       </c>
-      <c r="H30" s="28" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>docs/AGENTS.md (chatbot Swiggy tools section)</t>
         </is>
       </c>
-      <c r="I30" s="19" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="J30" s="25" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="K30" s="27" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L30" s="27" t="n"/>
-      <c r="M30" s="27" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="N30" s="29" t="n">
+      <c r="N31" t="n">
         <v>0</v>
       </c>
-      <c r="O30" s="28" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>P6-S04, P6-S01</t>
         </is>
       </c>
-      <c r="P30" s="28" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>NEEDS: OAuth token (read-only). All 3 tools callable from /chat; correct Swiggy data returned; graceful None on Swiggy failure; tool names appear in Groq tool_calls response.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="52.05" customHeight="1" s="81">
-      <c r="A31" s="31" t="inlineStr">
-        <is>
-          <t>WEEK 5 — Action Layer: Execution + Approval Gates</t>
-        </is>
-      </c>
-      <c r="B31" s="78" t="n"/>
-      <c r="C31" s="78" t="n"/>
-      <c r="D31" s="78" t="n"/>
-      <c r="E31" s="78" t="n"/>
-      <c r="F31" s="78" t="n"/>
-      <c r="G31" s="78" t="n"/>
-      <c r="H31" s="78" t="n"/>
-      <c r="I31" s="78" t="n"/>
-      <c r="J31" s="78" t="n"/>
-      <c r="K31" s="78" t="n"/>
-      <c r="L31" s="78" t="n"/>
-      <c r="M31" s="78" t="n"/>
-      <c r="N31" s="78" t="n"/>
-      <c r="O31" s="78" t="n"/>
-      <c r="P31" s="79" t="n"/>
-    </row>
     <row r="32" ht="6" customHeight="1" s="81">
-      <c r="A32" s="32" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="B32" s="32" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>P6-F04</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>feature/swiggy-frontend-connectors</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>/connectors page — data source management</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>New route /connectors. Lists connectors with status badges (Connected/Disconnected/Error). Shows last sync time, records synced, data freshness. Connect button triggers OAuth flow. Disconnect revokes token. Error state shows last error + reconnect. Works for Swiggy + future POS connector.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>feat: /connectors page — platform data source management with OAuth connect flow</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>None (frontend only)</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>P6-S01</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Can build now — reads from connectors table (already exists via P6-S02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="81">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>P6-F06</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>feature/swiggy-frontend-market</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Dashboard enhancements</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Add to existing dashboard: connector status widget (data source health bar), brief mode trigger button, today's Swiggy KPIs (orders today, delivery rating, top Swiggy seller), data_sources column on /runs list.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>feat: dashboard — connector status widget, brief trigger, live Swiggy KPIs, data_sources on runs list</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>None (frontend only)</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>P6-S01</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Can build now — connector status widget reads connectors table</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="52.05" customHeight="1" s="81">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>P6-S14</t>
         </is>
       </c>
-      <c r="C32" s="33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>feature/swiggy-action-queue</t>
         </is>
       </c>
-      <c r="D32" s="33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="E32" s="33" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>ActionQueueService + action_queue table</t>
         </is>
       </c>
-      <c r="F32" s="33" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>New table: id, org_id, action_type (AUTO/APPROVE_REQUIRED/RECOMMENDATION), payload jsonb, status (PENDING/APPROVED/EXECUTED/REJECTED/EXPIRED), approved_by, executed_at, error. ActionQueueService CRUD. Plan output includes action_queue section in API response.</t>
         </is>
       </c>
-      <c r="G32" s="33" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>feat: ActionQueueService + action_queue table — 3-tier action model with approval lifecycle</t>
         </is>
       </c>
-      <c r="H32" s="33" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>docs/ACTION_QUEUE.md (new), docs/APIS.md (action queue endpoints), docs/DECISIONS.md (D-021)</t>
         </is>
       </c>
-      <c r="I32" s="19" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="J32" s="25" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="K32" s="32" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L32" s="32" t="n"/>
-      <c r="M32" s="32" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="N32" s="34" t="n">
+      <c r="N34" t="n">
         <v>0</v>
       </c>
-      <c r="O32" s="33" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>P6-S10</t>
         </is>
       </c>
-      <c r="P32" s="33" t="inlineStr">
+      <c r="P34" t="inlineStr">
         <is>
           <t>No staging creds needed — action queue is pure backend, no Swiggy write calls yet.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1" s="81">
-      <c r="A33" s="27" t="inlineStr">
+    <row r="35" ht="52.05" customHeight="1" s="81">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>P6-F01</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>feature/swiggy-frontend-market</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Market intelligence panel (planning results page)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>New panel on /runs/{id}. Competitor pricing table: your price vs area avg vs cheapest competitor per dish category. Area occupancy badge (HIGH/MEDIUM/LOW). Instamart prices for shortage items. Pricing alerts (red if &gt;20% above area avg). Hidden when market_intel_output absent.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>feat: market intelligence panel — competitor pricing + area occupancy on planning results</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>None (frontend only)</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>P6-S10</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Depends on P6-S11 (market_intel_output in plan API response)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="52.05" customHeight="1" s="81">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>P7-S04</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>feature/ai-upgrades</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Structured outputs — tool_choice=required, zero JSON hallucination</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Upgrade chatbot Groq calls to tool_choice=required + strict JSON schema. Apply to all 3 Swiggy chatbot tools (search_menu, get_food_orders, search_products). Chatbot function calls never hallucinate JSON. Zero model coupling — works on any provider.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>feat: structured outputs — tool_choice=required across all chatbot tools</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>P6-F01</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Schema validation test; chatbot returns valid JSON on 10 consecutive calls</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="6" customHeight="1" s="81">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>RECORD END-TO-END DEMO HERE — chatbot + connectors + market intel + action queue all live</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="81">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>AI UPGRADES — strengthens job and investor story</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="52.05" customHeight="1" s="81">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>P7-S01</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>feature/ai-upgrades</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Prompt caching — 60-90% cost reduction on critic + aggregator</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Add Anthropic prompt caching headers to critic and aggregator LLM calls. Both have long system prompts repeated every run. Expected saving: 60-90% of prompt token cost per planning run. Graceful fallback on cache miss. Compatible with Google Gemini too.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>feat: prompt caching — cut LLM costs 80% on critic and aggregator nodes</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>docs/ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>P7-S04</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Cost log shows cache_hit=true on second run of same scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="52.05" customHeight="1" s="81">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>P7-S02</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>feature/ai-upgrades</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Reasoning model for critic — extended thinking, deeper plan evaluation</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Route critic node to Claude Opus with extended_thinking or o1/o3 via CometAPI. Critic reasons step-by-step before scoring — catches plan contradictions Sonnet misses. Falls back to Sonnet if reasoning model unavailable. One config flag: CRITIC_USE_REASONING=true. Zero coupling — model swapped via existing CometAPI registry.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>feat: reasoning model critic — extended thinking for deeper plan evaluation</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md, docs/DECISIONS.md</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>P7-S01</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Critic verdict quality test on 3 edge-case plans; reasoning chain logged</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="6" customHeight="1" s="81">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>P7-S05</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>feature/workflow-system</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Restaurant workflow system — owner-defined trigger-condition-action automations</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>New table: workflows (org_id, trigger, condition_json, action_type, action_payload, active). Triggers: AFTER_PLANNING_RUN, DAILY_BRIEF, ON_THRESHOLD. Actions: SEND_WHATSAPP, QUEUE_ACTION, CALL_WEBHOOK. WorkflowEngine evaluates conditions post-run and fires actions. /workflows UI page. Turns CortexKitchen from a tool into an OS.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>feat: workflow system — restaurant owners define custom automations</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>docs/ARCHITECTURE.md, docs/APIS.md</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>P7-S02</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>End-to-end: planning run fires whatsapp trigger; webhook called on threshold breach</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="81">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PRODUCT COMPLETENESS — brief, live monitor, MCP, debate, voice, remaining frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="52.05" customHeight="1" s="81">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>P6-S17</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>feature/swiggy-brief-mode</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BriefingService — automated 7am daily brief</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>APScheduler job at 07:00 IST per org. Lightweight run: demand_forecast + market_intel_node only. Pulls overnight Swiggy signals (get_food_orders since last run, track_food_order performance). Generates daily_brief JSON. Stores in daily_briefs table. Email digest (extends P5-11).</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>feat: BriefingService — automated daily morning brief with overnight Swiggy signals</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>docs/PRODUCT_MODES.md (new, brief mode), docs/APIS.md (brief endpoints)</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>P6-S10</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Scheduler fires at correct time; brief generates without full pipeline; daily_briefs row created; email sends</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="52.05" customHeight="1" s="81">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>P6-S18</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>feature/swiggy-live-mode</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LiveMonitorService — SSE feed during service hours</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>APScheduler-managed SSE stream active 12:00-14:00 and 19:00-22:00 IST. Polls every 30s: get_food_orders (activeOnly=true) for active delivery orders, track_food_order for in-flight ETAs, track_order for Instamart procurement status. Pushes events to /live page frontend. Alerts on: delivery &gt; SLA threshold, order spike, ingredient delivery confirmed.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>feat: LiveMonitorService — real-time Swiggy SSE during service hours (orders + procurement)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>docs/PRODUCT_MODES.md (live monitor section)</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>P6-S17, P6-S15</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SSE stream active only during service hours IST; events emitted on each 30s poll; delivery threshold alert fires; stream stops outside service window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="52.05" customHeight="1" s="81">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>P6-S19</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>feature/swiggy-mcp-tools</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>3 new CortexKitchen MCP server tools</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Add to mcp_server.py: get_market_brief (calls MarketIntelService live, returns competitor snapshot for Claude Desktop), get_action_queue (pending actions awaiting approval), approve_action (owner approves from Claude Desktop, triggers execution). JWT auth on all 3.</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>feat: 3 new MCP tools — get_market_brief, get_action_queue, approve_action</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>docs/APIS.md (MCP tools section), docs/ARCHITECTURE.md (MCP server updated)</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>P6-S14</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>All 3 tools smoke-tested in Claude Desktop; approve_action triggers execution end-to-end; JWT enforced</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="52.05" customHeight="1" s="81">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>P7-S03</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>feature/ai-upgrades</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Multi-agent debate critic — two critic instances, consensus scoring</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Run two LLM critic instances with opposing system prompts (optimistic vs conservative). Structured debate: each scores the plan, flags disagreements, moderator LLM resolves. Final verdict is consensus or flagged-disagreement. Provably better plan quality than single critic. Zero model coupling.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>feat: multi-agent debate critic — consensus scoring, catches more edge cases</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>P7-S05</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Debate resolves on 5 test plans; disagreement cases escalate correctly</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="52.05" customHeight="1" s="81">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>P6-R02</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>feature/swiggy-voice-interface</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Voice interface — Whisper + RAG chatbot</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Whisper transcription on browser-recorded question (MediaRecorder API). RAG chatbot (P5-12) answers. TTS reads back. Manager asks questions while walking the floor. Works with both synthetic and real Swiggy data now in DB. Blocked on P5-12 (already done).</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>feat: voice interface — Whisper transcription + RAG answer + TTS readback</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>docs/PRODUCT_MODES.md (voice section)</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>P6-S16</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Transcription accuracy smoke test; end-to-end voice → RAG answer → TTS; works with real Swiggy data in DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="52.05" customHeight="1" s="81">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>P6-F02</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>feature/swiggy-frontend-actions</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Action queue UI + procurement tracker</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>New section below plan output. Lists pending actions with type badge. Approve/Reject buttons for APPROVE_REQUIRED. Instamart cart preview modal (items, total, ETA) before approving checkout. Procurement tracker in inventory panel: placed orders, status, ETA.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>feat: action queue UI — approve/reject with cart preview, procurement tracker</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>None (frontend only)</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>P6-S13</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Depends on P6-S14 (action_queue in plan API response)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="6" customHeight="1" s="81">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>P6-F03</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>feature/swiggy-frontend-brief</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>/brief page — daily morning briefing</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>New route /brief. Overnight Swiggy performance (orders, avg delivery time, late %), today's demand forecast vs yesterday, top 3 action priorities, market snapshot. Auto-refreshes if brief is stale. Empty state when no brief yet.</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>feat: /brief page — daily morning operational briefing</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>None (frontend only)</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>P6-S16</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Depends on P6-S17 (BriefingService)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1" s="81">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>P6-F05</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>feature/swiggy-frontend-live</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>/live page — real-time service monitor</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S18). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>feat: /live page — SSE kitchen display for active orders and procurement tracking</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>None (frontend only)</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>P6-S18</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>SSE events render in real time; ETA countdown ticks; alert banner fires on delivery spike; Swiggy branding visible; inactive state shown outside service hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="52.05" customHeight="1" s="81">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BLOCKED — needs Swiggy staging creds for write tools</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="52.05" customHeight="1" s="81">
+      <c r="A52" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="B33" s="27" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>P6-S15</t>
         </is>
       </c>
-      <c r="C33" s="28" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>feature/swiggy-action-queue</t>
         </is>
       </c>
-      <c r="D33" s="28" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="E33" s="28" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>ProcurementExecutor — Instamart checkout flow</t>
         </is>
       </c>
-      <c r="F33" s="28" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Create executor/procurement.py. Flow: get_cart -&gt; clear_cart -&gt; update_cart([{spinId, qty}]) -&gt; get_cart (verify bill) -&gt; LangGraph interrupt() for owner approval -&gt; checkout (COD, Rs.999 cap). NON-IDEMPOTENT: on any 5xx from checkout, call get_orders before retrying — never blind-retry. Stores confirmed order in procurement_orders table. spinIds sourced from ProcurementEnricher state (P6-S09).</t>
         </is>
       </c>
-      <c r="G33" s="28" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>feat: ProcurementExecutor — Instamart checkout with LangGraph interrupt + check-then-retry safety</t>
         </is>
       </c>
-      <c r="H33" s="28" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>docs/SWIGGY_INTEGRATION.md (P6-S15 executor section)</t>
         </is>
       </c>
-      <c r="I33" s="19" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="J33" s="25" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="K33" s="27" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L33" s="27" t="n"/>
-      <c r="M33" s="27" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="N33" s="29" t="n">
+      <c r="N52" t="n">
         <v>0</v>
       </c>
-      <c r="O33" s="28" t="inlineStr">
+      <c r="O52" t="inlineStr">
         <is>
           <t>P6-S14, P6-S09</t>
         </is>
       </c>
-      <c r="P33" s="28" t="inlineStr">
+      <c r="P52" t="inlineStr">
         <is>
           <t>BLOCKED: needs staging creds (mcp-staging.swiggy.com). Check-then-retry fires on 5xx mock; LangGraph interrupt() pauses graph; cart verified before checkout; duplicate order prevention tested.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="52.05" customHeight="1" s="81">
-      <c r="A34" s="32" t="inlineStr">
+    <row r="53" ht="52.05" customHeight="1" s="81">
+      <c r="A53" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="B34" s="32" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>P6-S16</t>
         </is>
       </c>
-      <c r="C34" s="33" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>feature/swiggy-action-queue</t>
         </is>
       </c>
-      <c r="D34" s="33" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="E34" s="33" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>Dineout table booking execution</t>
         </is>
       </c>
-      <c r="F34" s="33" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>When dineout_manager_node queues book_table and owner approves: create_cart (DEAL_TICKET_PURCHASE) → book_table (slotId, itemId, reservationTime, guestCount, lat/lng). On 5xx: get_booking_status before retry. Confirmation written to reservations table.</t>
         </is>
       </c>
-      <c r="G34" s="33" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>feat: Dineout table booking execution with approval gate</t>
         </is>
       </c>
-      <c r="H34" s="33" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>docs/SWIGGY_INTEGRATION.md (book_table non-idempotency), docs/ACTION_QUEUE.md</t>
         </is>
       </c>
-      <c r="I34" s="20" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="J34" s="30" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K34" s="32" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L34" s="32" t="n"/>
-      <c r="M34" s="32" t="inlineStr">
+      <c r="M53" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="N34" s="34" t="n">
+      <c r="N53" t="n">
         <v>0</v>
       </c>
-      <c r="O34" s="33" t="inlineStr">
+      <c r="O53" t="inlineStr">
         <is>
           <t>P6-S14</t>
         </is>
       </c>
-      <c r="P34" s="33" t="inlineStr">
+      <c r="P53" t="inlineStr">
         <is>
           <t>BLOCKED: needs staging creds. book_table is a WRITE tool — places real Dineout bookings. Wait for mcp-staging.swiggy.com credentials before building.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="52.05" customHeight="1" s="81"/>
-    <row r="36" ht="52.05" customHeight="1" s="81">
-      <c r="A36" s="88" t="inlineStr">
-        <is>
-          <t>WEEK 6 — Product Modes: Brief, Live, MCP Expansion</t>
-        </is>
-      </c>
-      <c r="B36" s="78" t="n"/>
-      <c r="C36" s="78" t="n"/>
-      <c r="D36" s="78" t="n"/>
-      <c r="E36" s="78" t="n"/>
-      <c r="F36" s="78" t="n"/>
-      <c r="G36" s="78" t="n"/>
-      <c r="H36" s="78" t="n"/>
-      <c r="I36" s="78" t="n"/>
-      <c r="J36" s="78" t="n"/>
-      <c r="K36" s="78" t="n"/>
-      <c r="L36" s="78" t="n"/>
-      <c r="M36" s="78" t="n"/>
-      <c r="N36" s="78" t="n"/>
-      <c r="O36" s="78" t="n"/>
-      <c r="P36" s="79" t="n"/>
-    </row>
-    <row r="37" ht="6" customHeight="1" s="81">
-      <c r="A37" s="36" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B37" s="36" t="inlineStr">
-        <is>
-          <t>P6-S17</t>
-        </is>
-      </c>
-      <c r="C37" s="37" t="inlineStr">
-        <is>
-          <t>feature/swiggy-brief-mode</t>
-        </is>
-      </c>
-      <c r="D37" s="37" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="E37" s="37" t="inlineStr">
-        <is>
-          <t>BriefingService — automated 7am daily brief</t>
-        </is>
-      </c>
-      <c r="F37" s="37" t="inlineStr">
-        <is>
-          <t>APScheduler job at 07:00 IST per org. Lightweight run: demand_forecast + market_intel_node only. Pulls overnight Swiggy signals (get_food_orders since last run, track_food_order performance). Generates daily_brief JSON. Stores in daily_briefs table. Email digest (extends P5-11).</t>
-        </is>
-      </c>
-      <c r="G37" s="37" t="inlineStr">
-        <is>
-          <t>feat: BriefingService — automated daily morning brief with overnight Swiggy signals</t>
-        </is>
-      </c>
-      <c r="H37" s="37" t="inlineStr">
-        <is>
-          <t>docs/PRODUCT_MODES.md (new, brief mode), docs/APIS.md (brief endpoints)</t>
-        </is>
-      </c>
-      <c r="I37" s="19" t="inlineStr">
+    <row r="54" ht="36.6" customHeight="1" s="81">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>P7-S07</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>feature/computer-use</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Computer use agent — automate Swiggy Partner Dashboard</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Claude computer-use agent automates Swiggy Partner Dashboard actions not exposed via MCP: menu price updates, promo activation, opening delivery hours. Triggered from action queue. Sandboxed browser session. Claude-specific today; fallback to manual action link if unavailable.</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>feat: computer use — automate Swiggy Partner Dashboard actions</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>docs/ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="J37" s="30" t="inlineStr">
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>P7-S03</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Computer use agent updates one menu price end-to-end in sandbox</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1" s="81">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DOCS + PHASE 6 MILESTONE MERGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="52.05" customHeight="1" s="81">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>P6-D01</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>feature/swiggy-docs</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>5 new documentation files</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>CONNECTORS.md: BaseConnector interface, sync vs enrich, how to add new connector. SWIGGY_INTEGRATION.md: all 22 tools, parameter mappings, OAuth, rate limits, error handling. ACTION_QUEUE.md: action types, approval flow, non-idempotent patterns. DATA_SOURCES.md: all sources, channels, sync frequency. PRODUCT_MODES.md: ops/brief/live/voice mode specs.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>docs: 5 new documentation files for Phase 6 connector + action + product mode layer</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>docs/CONNECTORS.md, docs/SWIGGY_INTEGRATION.md, docs/ACTION_QUEUE.md, docs/DATA_SOURCES.md, docs/PRODUCT_MODES.md</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>P6-F06</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>All 5 files present; no broken links; tool parameter tables accurate vs Swiggy docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="52.05" customHeight="1" s="81">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>P6-D02</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>feature/swiggy-docs</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Update CLAUDE.md, README.md, Swiggy deep-dive for Phase 6 completion</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>CLAUDE.md: update Current system state to Phase 6 complete (11-node pipeline, 22 Swiggy tools, full action + brief + live layer). README.md: add Phase 6 achievements, Swiggy integration summary, demo instructions. CortexKitchen_Swiggy_Deep_Dive.html: mark all chapters complete, update progress bar to 100%.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>docs: Phase 6 milestone — CLAUDE.md, README, Swiggy deep-dive final update</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>CLAUDE.md, README.md, CortexKitchen_Swiggy_Deep_Dive.html</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>P6-D01</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>CLAUDE.md system state accurate; README demo instructions work end-to-end; deep-dive HTML shows 100% progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="52.05" customHeight="1" s="81">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>P6-D03</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>dev -&gt; main PR</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Phase 6 milestone merge to main</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Merge feature/ck-v2-platform → dev → main. All 11 nodes verified in LangSmith. All 22 Swiggy tools exercised in staging. POS connector imports CSV end-to-end. Voice interface smoke tested. Action queue end-to-end. All 3 product modes verified. 5 new frontend pages smoke tested. Full test suite green.</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>release: Phase 6 complete — CortexKitchen v2 Swiggy-native restaurant OS</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>README.md (portfolio headline), docs/ROADMAP.md (Phase 6 complete)</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>P6-D02</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Full test suite green; 11 nodes in LangSmith; staging demo clean; portfolio README updated; docs website prep checklist done</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="52.05" customHeight="1" s="81">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>PHASE 7 — Production, CI/CD, Public Release</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="52.05" customHeight="1" s="81">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>P7-01</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>feature/phase7-cicd</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>CI/CD — GitHub Actions</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Automated on every PR: unit + integration + RAGAS evals + DeepEval; lint; type check; frontend build; coverage report. Fail on critic score regression. Cache pip dependencies.</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>feat: CI/CD — automated test + eval pipeline on every PR</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>docs/ROADMAP.md</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>P6-D03</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>CI passes on clean repo; fails on intentional test break; eval regression detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="6" customHeight="1" s="81">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>P7-02</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>feature/phase7-cloud-deploy</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Cloud deployment — Railway / Fly.io</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Containerise API + frontend. Deploy to Railway or Fly.io. Managed Postgres + Redis + Qdrant. Production env vars. Swiggy OAuth redirect URI updated for production domain. Health endpoint green on production URL.</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>feat: cloud deployment — production on Railway/Fly.io</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>docs/ROADMAP.md</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>P7-01</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Production URL health check green; all env vars; Swiggy OAuth works on production domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="66" customHeight="1" s="81">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>P7-03</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>feature/phase7-prod-hardening</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Production hardening</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Rate limiting (slowapi). Secrets management (not env file). CORS lockdown. JWT key rotation. Sentry alerts tuned for production. Load test with k6.</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>feat: production hardening — rate limiting, secrets, CORS, JWT rotation</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>docs/ROADMAP.md</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K37" s="36" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L37" s="36" t="n"/>
-      <c r="M37" s="36" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="N37" s="38" t="n">
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
         <v>0</v>
       </c>
-      <c r="O37" s="37" t="inlineStr">
-        <is>
-          <t>P6-S10</t>
-        </is>
-      </c>
-      <c r="P37" s="37" t="inlineStr">
-        <is>
-          <t>Scheduler fires at correct time; brief generates without full pipeline; daily_briefs row created; email sends</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1" s="81">
-      <c r="A38" s="27" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B38" s="27" t="inlineStr">
-        <is>
-          <t>P6-S18</t>
-        </is>
-      </c>
-      <c r="C38" s="28" t="inlineStr">
-        <is>
-          <t>feature/swiggy-live-mode</t>
-        </is>
-      </c>
-      <c r="D38" s="28" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="E38" s="28" t="inlineStr">
-        <is>
-          <t>LiveMonitorService — SSE feed during service hours</t>
-        </is>
-      </c>
-      <c r="F38" s="28" t="inlineStr">
-        <is>
-          <t>APScheduler-managed SSE stream active 12:00-14:00 and 19:00-22:00 IST. Polls every 30s: get_food_orders (activeOnly=true) for active delivery orders, track_food_order for in-flight ETAs, track_order for Instamart procurement status. Pushes events to /live page frontend. Alerts on: delivery &gt; SLA threshold, order spike, ingredient delivery confirmed.</t>
-        </is>
-      </c>
-      <c r="G38" s="28" t="inlineStr">
-        <is>
-          <t>feat: LiveMonitorService — real-time Swiggy SSE during service hours (orders + procurement)</t>
-        </is>
-      </c>
-      <c r="H38" s="28" t="inlineStr">
-        <is>
-          <t>docs/PRODUCT_MODES.md (live monitor section)</t>
-        </is>
-      </c>
-      <c r="I38" s="19" t="inlineStr">
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>P7-02</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Rate limit smoke test; CORS rejection; Sentry alert fires on 500; k6 load test passes</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="39.6" customHeight="1" s="81">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>P7-04</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>feature/phase7-docs-website</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Mintlify docs website</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Point Mintlify at docs/ folder. Navigation: architecture, connectors, agents, API reference, Swiggy integration guide, evaluation, deployment. Custom domain. Public URL to share with Swiggy team, recruiters, restaurant clients.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>feat: Mintlify docs website — public-facing CortexKitchen v2 documentation</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>All docs/ files</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="J38" s="25" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K38" s="27" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L38" s="27" t="n"/>
-      <c r="M38" s="27" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="N38" s="29" t="n">
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
         <v>0</v>
       </c>
-      <c r="O38" s="28" t="inlineStr">
-        <is>
-          <t>P6-S17, P6-S15</t>
-        </is>
-      </c>
-      <c r="P38" s="28" t="inlineStr">
-        <is>
-          <t>SSE stream active only during service hours IST; events emitted on each 30s poll; delivery threshold alert fires; stream stops outside service window.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="52.05" customHeight="1" s="81">
-      <c r="A39" s="36" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B39" s="36" t="inlineStr">
-        <is>
-          <t>P6-S19</t>
-        </is>
-      </c>
-      <c r="C39" s="37" t="inlineStr">
-        <is>
-          <t>feature/swiggy-mcp-tools</t>
-        </is>
-      </c>
-      <c r="D39" s="37" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="E39" s="37" t="inlineStr">
-        <is>
-          <t>3 new CortexKitchen MCP server tools</t>
-        </is>
-      </c>
-      <c r="F39" s="37" t="inlineStr">
-        <is>
-          <t>Add to mcp_server.py: get_market_brief (calls MarketIntelService live, returns competitor snapshot for Claude Desktop), get_action_queue (pending actions awaiting approval), approve_action (owner approves from Claude Desktop, triggers execution). JWT auth on all 3.</t>
-        </is>
-      </c>
-      <c r="G39" s="37" t="inlineStr">
-        <is>
-          <t>feat: 3 new MCP tools — get_market_brief, get_action_queue, approve_action</t>
-        </is>
-      </c>
-      <c r="H39" s="37" t="inlineStr">
-        <is>
-          <t>docs/APIS.md (MCP tools section), docs/ARCHITECTURE.md (MCP server updated)</t>
-        </is>
-      </c>
-      <c r="I39" s="19" t="inlineStr">
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>P7-03</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Docs site live at public URL; all 13 doc files render; search works; no broken links</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>P7-05</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>dev -&gt; main PR</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Sync Phase 7 to main — public release</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Live production URL. README updated with live demo link + docs website link. Apply to jobs immediately. Update portfolio.</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>release: Phase 7 complete — CortexKitchen v2 live in production</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>README.md, anoushkavyas.vercel.app portfolio</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="J39" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K39" s="36" t="inlineStr">
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L39" s="36" t="n"/>
-      <c r="M39" s="36" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="N39" s="38" t="n">
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
         <v>0</v>
       </c>
-      <c r="O39" s="37" t="inlineStr">
-        <is>
-          <t>P6-S14</t>
-        </is>
-      </c>
-      <c r="P39" s="37" t="inlineStr">
-        <is>
-          <t>All 3 tools smoke-tested in Claude Desktop; approve_action triggers execution end-to-end; JWT enforced</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="52.05" customHeight="1" s="81"/>
-    <row r="41" ht="6" customHeight="1" s="81">
-      <c r="A41" s="83" t="inlineStr">
-        <is>
-          <t>WEEK 6-7 — Original P6 Tasks (POS Connector + Voice)</t>
-        </is>
-      </c>
-      <c r="B41" s="78" t="n"/>
-      <c r="C41" s="78" t="n"/>
-      <c r="D41" s="78" t="n"/>
-      <c r="E41" s="78" t="n"/>
-      <c r="F41" s="78" t="n"/>
-      <c r="G41" s="78" t="n"/>
-      <c r="H41" s="78" t="n"/>
-      <c r="I41" s="78" t="n"/>
-      <c r="J41" s="78" t="n"/>
-      <c r="K41" s="78" t="n"/>
-      <c r="L41" s="78" t="n"/>
-      <c r="M41" s="78" t="n"/>
-      <c r="N41" s="78" t="n"/>
-      <c r="O41" s="78" t="n"/>
-      <c r="P41" s="79" t="n"/>
-    </row>
-    <row r="42" ht="18" customHeight="1" s="81">
-      <c r="A42" s="77" t="n"/>
-      <c r="B42" s="78" t="n"/>
-      <c r="C42" s="78" t="n"/>
-      <c r="D42" s="78" t="n"/>
-      <c r="E42" s="78" t="n"/>
-      <c r="F42" s="78" t="n"/>
-      <c r="G42" s="78" t="n"/>
-      <c r="H42" s="78" t="n"/>
-      <c r="I42" s="78" t="n"/>
-      <c r="J42" s="78" t="n"/>
-      <c r="K42" s="78" t="n"/>
-      <c r="L42" s="78" t="n"/>
-      <c r="M42" s="78" t="n"/>
-      <c r="N42" s="78" t="n"/>
-      <c r="O42" s="78" t="n"/>
-      <c r="P42" s="79" t="n"/>
-    </row>
-    <row r="43" ht="52.05" customHeight="1" s="81">
-      <c r="A43" s="22" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B43" s="22" t="inlineStr">
-        <is>
-          <t>P6-R02</t>
-        </is>
-      </c>
-      <c r="C43" s="23" t="inlineStr">
-        <is>
-          <t>feature/swiggy-voice-interface</t>
-        </is>
-      </c>
-      <c r="D43" s="23" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="E43" s="23" t="inlineStr">
-        <is>
-          <t>Voice interface — Whisper + RAG chatbot</t>
-        </is>
-      </c>
-      <c r="F43" s="23" t="inlineStr">
-        <is>
-          <t>Whisper transcription on browser-recorded question (MediaRecorder API). RAG chatbot (P5-12) answers. TTS reads back. Manager asks questions while walking the floor. Works with both synthetic and real Swiggy data now in DB. Blocked on P5-12 (already done).</t>
-        </is>
-      </c>
-      <c r="G43" s="23" t="inlineStr">
-        <is>
-          <t>feat: voice interface — Whisper transcription + RAG answer + TTS readback</t>
-        </is>
-      </c>
-      <c r="H43" s="23" t="inlineStr">
-        <is>
-          <t>docs/PRODUCT_MODES.md (voice section)</t>
-        </is>
-      </c>
-      <c r="I43" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J43" s="19" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K43" s="22" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L43" s="22" t="n"/>
-      <c r="M43" s="22" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="N43" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O43" s="23" t="inlineStr">
-        <is>
-          <t>P6-S16</t>
-        </is>
-      </c>
-      <c r="P43" s="23" t="inlineStr">
-        <is>
-          <t>Transcription accuracy smoke test; end-to-end voice → RAG answer → TTS; works with real Swiggy data in DB</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="52.05" customHeight="1" s="81"/>
-    <row r="45" ht="52.05" customHeight="1" s="81">
-      <c r="A45" s="82" t="inlineStr">
-        <is>
-          <t>WEEK 7 — Frontend: 5 New Pages + 3 New Panels</t>
-        </is>
-      </c>
-      <c r="B45" s="78" t="n"/>
-      <c r="C45" s="78" t="n"/>
-      <c r="D45" s="78" t="n"/>
-      <c r="E45" s="78" t="n"/>
-      <c r="F45" s="78" t="n"/>
-      <c r="G45" s="78" t="n"/>
-      <c r="H45" s="78" t="n"/>
-      <c r="I45" s="78" t="n"/>
-      <c r="J45" s="78" t="n"/>
-      <c r="K45" s="78" t="n"/>
-      <c r="L45" s="78" t="n"/>
-      <c r="M45" s="78" t="n"/>
-      <c r="N45" s="78" t="n"/>
-      <c r="O45" s="78" t="n"/>
-      <c r="P45" s="79" t="n"/>
-    </row>
-    <row r="46" ht="52.05" customHeight="1" s="81">
-      <c r="A46" s="17" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B46" s="17" t="inlineStr">
-        <is>
-          <t>P6-F01</t>
-        </is>
-      </c>
-      <c r="C46" s="18" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-market</t>
-        </is>
-      </c>
-      <c r="D46" s="18" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="E46" s="18" t="inlineStr">
-        <is>
-          <t>Market intelligence panel (planning results page)</t>
-        </is>
-      </c>
-      <c r="F46" s="18" t="inlineStr">
-        <is>
-          <t>New panel on /runs/{id}. Competitor pricing table: your price vs area avg vs cheapest competitor per dish category. Area occupancy badge (HIGH/MEDIUM/LOW). Instamart prices for shortage items. Pricing alerts (red if &gt;20% above area avg). Hidden when market_intel_output absent.</t>
-        </is>
-      </c>
-      <c r="G46" s="18" t="inlineStr">
-        <is>
-          <t>feat: market intelligence panel — competitor pricing + area occupancy on planning results</t>
-        </is>
-      </c>
-      <c r="H46" s="18" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="I46" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J46" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K46" s="17" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L46" s="17" t="n"/>
-      <c r="M46" s="17" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="N46" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O46" s="18" t="inlineStr">
-        <is>
-          <t>P6-S10</t>
-        </is>
-      </c>
-      <c r="P46" s="18" t="inlineStr">
-        <is>
-          <t>Depends on P6-S11 (market_intel_output in plan API response)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="52.05" customHeight="1" s="81">
-      <c r="A47" s="22" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B47" s="22" t="inlineStr">
-        <is>
-          <t>P6-F02</t>
-        </is>
-      </c>
-      <c r="C47" s="23" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-actions</t>
-        </is>
-      </c>
-      <c r="D47" s="23" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="E47" s="23" t="inlineStr">
-        <is>
-          <t>Action queue UI + procurement tracker</t>
-        </is>
-      </c>
-      <c r="F47" s="23" t="inlineStr">
-        <is>
-          <t>New section below plan output. Lists pending actions with type badge. Approve/Reject buttons for APPROVE_REQUIRED. Instamart cart preview modal (items, total, ETA) before approving checkout. Procurement tracker in inventory panel: placed orders, status, ETA.</t>
-        </is>
-      </c>
-      <c r="G47" s="23" t="inlineStr">
-        <is>
-          <t>feat: action queue UI — approve/reject with cart preview, procurement tracker</t>
-        </is>
-      </c>
-      <c r="H47" s="23" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="I47" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J47" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K47" s="22" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L47" s="22" t="n"/>
-      <c r="M47" s="22" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="N47" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O47" s="23" t="inlineStr">
-        <is>
-          <t>P6-S13</t>
-        </is>
-      </c>
-      <c r="P47" s="23" t="inlineStr">
-        <is>
-          <t>Depends on P6-S14 (action_queue in plan API response)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="52.05" customHeight="1" s="81">
-      <c r="A48" s="17" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B48" s="17" t="inlineStr">
-        <is>
-          <t>P6-F03</t>
-        </is>
-      </c>
-      <c r="C48" s="18" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-brief</t>
-        </is>
-      </c>
-      <c r="D48" s="18" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="E48" s="18" t="inlineStr">
-        <is>
-          <t>/brief page — daily morning briefing</t>
-        </is>
-      </c>
-      <c r="F48" s="18" t="inlineStr">
-        <is>
-          <t>New route /brief. Overnight Swiggy performance (orders, avg delivery time, late %), today's demand forecast vs yesterday, top 3 action priorities, market snapshot. Auto-refreshes if brief is stale. Empty state when no brief yet.</t>
-        </is>
-      </c>
-      <c r="G48" s="18" t="inlineStr">
-        <is>
-          <t>feat: /brief page — daily morning operational briefing</t>
-        </is>
-      </c>
-      <c r="H48" s="18" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="I48" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J48" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K48" s="17" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L48" s="17" t="n"/>
-      <c r="M48" s="17" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="N48" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O48" s="18" t="inlineStr">
-        <is>
-          <t>P6-S16</t>
-        </is>
-      </c>
-      <c r="P48" s="18" t="inlineStr">
-        <is>
-          <t>Depends on P6-S17 (BriefingService)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="6" customHeight="1" s="81">
-      <c r="A49" s="22" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B49" s="22" t="inlineStr">
-        <is>
-          <t>P6-F04</t>
-        </is>
-      </c>
-      <c r="C49" s="23" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-connectors</t>
-        </is>
-      </c>
-      <c r="D49" s="23" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="E49" s="23" t="inlineStr">
-        <is>
-          <t>/connectors page — data source management</t>
-        </is>
-      </c>
-      <c r="F49" s="23" t="inlineStr">
-        <is>
-          <t>New route /connectors. Lists connectors with status badges (Connected/Disconnected/Error). Shows last sync time, records synced, data freshness. Connect button triggers OAuth flow. Disconnect revokes token. Error state shows last error + reconnect. Works for Swiggy + future POS connector.</t>
-        </is>
-      </c>
-      <c r="G49" s="23" t="inlineStr">
-        <is>
-          <t>feat: /connectors page — platform data source management with OAuth connect flow</t>
-        </is>
-      </c>
-      <c r="H49" s="23" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="I49" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J49" s="30" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="K49" s="22" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L49" s="22" t="n"/>
-      <c r="M49" s="22" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="N49" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O49" s="23" t="inlineStr">
-        <is>
-          <t>P6-S01</t>
-        </is>
-      </c>
-      <c r="P49" s="23" t="inlineStr">
-        <is>
-          <t>Can build now — reads from connectors table (already exists via P6-S02)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1" s="81">
-      <c r="A50" s="27" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B50" s="27" t="inlineStr">
-        <is>
-          <t>P6-F05</t>
-        </is>
-      </c>
-      <c r="C50" s="28" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-live</t>
-        </is>
-      </c>
-      <c r="D50" s="28" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="E50" s="28" t="inlineStr">
-        <is>
-          <t>/live page — real-time service monitor</t>
-        </is>
-      </c>
-      <c r="F50" s="28" t="inlineStr">
-        <is>
-          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S18). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
-        </is>
-      </c>
-      <c r="G50" s="28" t="inlineStr">
-        <is>
-          <t>feat: /live page — SSE kitchen display for active orders and procurement tracking</t>
-        </is>
-      </c>
-      <c r="H50" s="28" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="I50" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J50" s="25" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K50" s="27" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L50" s="27" t="n"/>
-      <c r="M50" s="27" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="N50" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O50" s="28" t="inlineStr">
-        <is>
-          <t>P6-S18</t>
-        </is>
-      </c>
-      <c r="P50" s="28" t="inlineStr">
-        <is>
-          <t>SSE events render in real time; ETA countdown ticks; alert banner fires on delivery spike; Swiggy branding visible; inactive state shown outside service hours.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="52.05" customHeight="1" s="81">
-      <c r="A51" s="22" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B51" s="22" t="inlineStr">
-        <is>
-          <t>P6-F06</t>
-        </is>
-      </c>
-      <c r="C51" s="23" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-market</t>
-        </is>
-      </c>
-      <c r="D51" s="23" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="E51" s="23" t="inlineStr">
-        <is>
-          <t>Dashboard enhancements</t>
-        </is>
-      </c>
-      <c r="F51" s="23" t="inlineStr">
-        <is>
-          <t>Add to existing dashboard: connector status widget (data source health bar), brief mode trigger button, today's Swiggy KPIs (orders today, delivery rating, top Swiggy seller), data_sources column on /runs list.</t>
-        </is>
-      </c>
-      <c r="G51" s="23" t="inlineStr">
-        <is>
-          <t>feat: dashboard — connector status widget, brief trigger, live Swiggy KPIs, data_sources on runs list</t>
-        </is>
-      </c>
-      <c r="H51" s="23" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="I51" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J51" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K51" s="22" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L51" s="22" t="n"/>
-      <c r="M51" s="22" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="N51" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O51" s="23" t="inlineStr">
-        <is>
-          <t>P6-S01</t>
-        </is>
-      </c>
-      <c r="P51" s="23" t="inlineStr">
-        <is>
-          <t>Can build now — connector status widget reads connectors table</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="52.05" customHeight="1" s="81"/>
-    <row r="53" ht="52.05" customHeight="1" s="81">
-      <c r="A53" s="88" t="inlineStr">
-        <is>
-          <t>WEEK 8 — Docs + Merge: Phase 6 Complete</t>
-        </is>
-      </c>
-      <c r="B53" s="78" t="n"/>
-      <c r="C53" s="78" t="n"/>
-      <c r="D53" s="78" t="n"/>
-      <c r="E53" s="78" t="n"/>
-      <c r="F53" s="78" t="n"/>
-      <c r="G53" s="78" t="n"/>
-      <c r="H53" s="78" t="n"/>
-      <c r="I53" s="78" t="n"/>
-      <c r="J53" s="78" t="n"/>
-      <c r="K53" s="78" t="n"/>
-      <c r="L53" s="78" t="n"/>
-      <c r="M53" s="78" t="n"/>
-      <c r="N53" s="78" t="n"/>
-      <c r="O53" s="78" t="n"/>
-      <c r="P53" s="79" t="n"/>
-    </row>
-    <row r="54" ht="36.6" customHeight="1" s="81">
-      <c r="A54" s="36" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B54" s="36" t="inlineStr">
-        <is>
-          <t>P6-D01</t>
-        </is>
-      </c>
-      <c r="C54" s="37" t="inlineStr">
-        <is>
-          <t>feature/swiggy-docs</t>
-        </is>
-      </c>
-      <c r="D54" s="37" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="E54" s="37" t="inlineStr">
-        <is>
-          <t>5 new documentation files</t>
-        </is>
-      </c>
-      <c r="F54" s="37" t="inlineStr">
-        <is>
-          <t>CONNECTORS.md: BaseConnector interface, sync vs enrich, how to add new connector. SWIGGY_INTEGRATION.md: all 22 tools, parameter mappings, OAuth, rate limits, error handling. ACTION_QUEUE.md: action types, approval flow, non-idempotent patterns. DATA_SOURCES.md: all sources, channels, sync frequency. PRODUCT_MODES.md: ops/brief/live/voice mode specs.</t>
-        </is>
-      </c>
-      <c r="G54" s="37" t="inlineStr">
-        <is>
-          <t>docs: 5 new documentation files for Phase 6 connector + action + product mode layer</t>
-        </is>
-      </c>
-      <c r="H54" s="37" t="inlineStr">
-        <is>
-          <t>docs/CONNECTORS.md, docs/SWIGGY_INTEGRATION.md, docs/ACTION_QUEUE.md, docs/DATA_SOURCES.md, docs/PRODUCT_MODES.md</t>
-        </is>
-      </c>
-      <c r="I54" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J54" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K54" s="36" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L54" s="36" t="n"/>
-      <c r="M54" s="36" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="N54" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="37" t="inlineStr">
-        <is>
-          <t>P6-F06</t>
-        </is>
-      </c>
-      <c r="P54" s="37" t="inlineStr">
-        <is>
-          <t>All 5 files present; no broken links; tool parameter tables accurate vs Swiggy docs</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1" s="81">
-      <c r="A55" s="27" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B55" s="27" t="inlineStr">
-        <is>
-          <t>P6-D02</t>
-        </is>
-      </c>
-      <c r="C55" s="28" t="inlineStr">
-        <is>
-          <t>feature/swiggy-docs</t>
-        </is>
-      </c>
-      <c r="D55" s="28" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="E55" s="28" t="inlineStr">
-        <is>
-          <t>Update CLAUDE.md, README.md, Swiggy deep-dive for Phase 6 completion</t>
-        </is>
-      </c>
-      <c r="F55" s="28" t="inlineStr">
-        <is>
-          <t>CLAUDE.md: update Current system state to Phase 6 complete (11-node pipeline, 22 Swiggy tools, full action + brief + live layer). README.md: add Phase 6 achievements, Swiggy integration summary, demo instructions. CortexKitchen_Swiggy_Deep_Dive.html: mark all chapters complete, update progress bar to 100%.</t>
-        </is>
-      </c>
-      <c r="G55" s="28" t="inlineStr">
-        <is>
-          <t>docs: Phase 6 milestone — CLAUDE.md, README, Swiggy deep-dive final update</t>
-        </is>
-      </c>
-      <c r="H55" s="28" t="inlineStr">
-        <is>
-          <t>CLAUDE.md, README.md, CortexKitchen_Swiggy_Deep_Dive.html</t>
-        </is>
-      </c>
-      <c r="I55" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J55" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K55" s="27" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L55" s="27" t="n"/>
-      <c r="M55" s="27" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="N55" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O55" s="28" t="inlineStr">
-        <is>
-          <t>P6-D01</t>
-        </is>
-      </c>
-      <c r="P55" s="28" t="inlineStr">
-        <is>
-          <t>CLAUDE.md system state accurate; README demo instructions work end-to-end; deep-dive HTML shows 100% progress.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="52.05" customHeight="1" s="81">
-      <c r="A56" s="36" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B56" s="36" t="inlineStr">
-        <is>
-          <t>P6-D03</t>
-        </is>
-      </c>
-      <c r="C56" s="37" t="inlineStr">
-        <is>
-          <t>dev -&gt; main PR</t>
-        </is>
-      </c>
-      <c r="D56" s="37" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="E56" s="37" t="inlineStr">
-        <is>
-          <t>Phase 6 milestone merge to main</t>
-        </is>
-      </c>
-      <c r="F56" s="37" t="inlineStr">
-        <is>
-          <t>Merge feature/ck-v2-platform → dev → main. All 11 nodes verified in LangSmith. All 22 Swiggy tools exercised in staging. POS connector imports CSV end-to-end. Voice interface smoke tested. Action queue end-to-end. All 3 product modes verified. 5 new frontend pages smoke tested. Full test suite green.</t>
-        </is>
-      </c>
-      <c r="G56" s="37" t="inlineStr">
-        <is>
-          <t>release: Phase 6 complete — CortexKitchen v2 Swiggy-native restaurant OS</t>
-        </is>
-      </c>
-      <c r="H56" s="37" t="inlineStr">
-        <is>
-          <t>README.md (portfolio headline), docs/ROADMAP.md (Phase 6 complete)</t>
-        </is>
-      </c>
-      <c r="I56" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J56" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="K56" s="36" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L56" s="36" t="n"/>
-      <c r="M56" s="36" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="N56" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="O56" s="37" t="inlineStr">
-        <is>
-          <t>P6-D02</t>
-        </is>
-      </c>
-      <c r="P56" s="37" t="inlineStr">
-        <is>
-          <t>Full test suite green; 11 nodes in LangSmith; staging demo clean; portfolio README updated; docs website prep checklist done</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="52.05" customHeight="1" s="81"/>
-    <row r="58" ht="52.05" customHeight="1" s="81">
-      <c r="A58" s="40" t="inlineStr">
-        <is>
-          <t>PHASE 7 — Production, CI/CD, Docs Website</t>
-        </is>
-      </c>
-      <c r="B58" s="78" t="n"/>
-      <c r="C58" s="78" t="n"/>
-      <c r="D58" s="78" t="n"/>
-      <c r="E58" s="78" t="n"/>
-      <c r="F58" s="78" t="n"/>
-      <c r="G58" s="78" t="n"/>
-      <c r="H58" s="78" t="n"/>
-      <c r="I58" s="78" t="n"/>
-      <c r="J58" s="78" t="n"/>
-      <c r="K58" s="78" t="n"/>
-      <c r="L58" s="78" t="n"/>
-      <c r="M58" s="78" t="n"/>
-      <c r="N58" s="78" t="n"/>
-      <c r="O58" s="78" t="n"/>
-      <c r="P58" s="79" t="n"/>
-    </row>
-    <row r="59" ht="52.05" customHeight="1" s="81">
-      <c r="A59" s="41" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B59" s="41" t="inlineStr">
-        <is>
-          <t>P7-01</t>
-        </is>
-      </c>
-      <c r="C59" s="42" t="inlineStr">
-        <is>
-          <t>feature/phase7-cicd</t>
-        </is>
-      </c>
-      <c r="D59" s="42" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="E59" s="42" t="inlineStr">
-        <is>
-          <t>CI/CD — GitHub Actions</t>
-        </is>
-      </c>
-      <c r="F59" s="42" t="inlineStr">
-        <is>
-          <t>Automated on every PR: unit + integration + RAGAS evals + DeepEval; lint; type check; frontend build; coverage report. Fail on critic score regression. Cache pip dependencies.</t>
-        </is>
-      </c>
-      <c r="G59" s="42" t="inlineStr">
-        <is>
-          <t>feat: CI/CD — automated test + eval pipeline on every PR</t>
-        </is>
-      </c>
-      <c r="H59" s="42" t="inlineStr">
-        <is>
-          <t>docs/ROADMAP.md</t>
-        </is>
-      </c>
-      <c r="I59" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J59" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K59" s="41" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L59" s="41" t="n"/>
-      <c r="M59" s="41" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="N59" s="43" t="n">
-        <v>0</v>
-      </c>
-      <c r="O59" s="42" t="inlineStr">
-        <is>
-          <t>P6-D03</t>
-        </is>
-      </c>
-      <c r="P59" s="42" t="inlineStr">
-        <is>
-          <t>CI passes on clean repo; fails on intentional test break; eval regression detected</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="52.05" customHeight="1" s="81">
-      <c r="A60" s="22" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B60" s="22" t="inlineStr">
-        <is>
-          <t>P7-02</t>
-        </is>
-      </c>
-      <c r="C60" s="23" t="inlineStr">
-        <is>
-          <t>feature/phase7-cloud-deploy</t>
-        </is>
-      </c>
-      <c r="D60" s="23" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="E60" s="23" t="inlineStr">
-        <is>
-          <t>Cloud deployment — Railway / Fly.io</t>
-        </is>
-      </c>
-      <c r="F60" s="23" t="inlineStr">
-        <is>
-          <t>Containerise API + frontend. Deploy to Railway or Fly.io. Managed Postgres + Redis + Qdrant. Production env vars. Swiggy OAuth redirect URI updated for production domain. Health endpoint green on production URL.</t>
-        </is>
-      </c>
-      <c r="G60" s="23" t="inlineStr">
-        <is>
-          <t>feat: cloud deployment — production on Railway/Fly.io</t>
-        </is>
-      </c>
-      <c r="H60" s="23" t="inlineStr">
-        <is>
-          <t>docs/ROADMAP.md</t>
-        </is>
-      </c>
-      <c r="I60" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J60" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K60" s="22" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L60" s="22" t="n"/>
-      <c r="M60" s="22" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="N60" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O60" s="23" t="inlineStr">
-        <is>
-          <t>P7-01</t>
-        </is>
-      </c>
-      <c r="P60" s="23" t="inlineStr">
-        <is>
-          <t>Production URL health check green; all env vars; Swiggy OAuth works on production domain</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="6" customHeight="1" s="81">
-      <c r="A61" s="41" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B61" s="41" t="inlineStr">
-        <is>
-          <t>P7-03</t>
-        </is>
-      </c>
-      <c r="C61" s="42" t="inlineStr">
-        <is>
-          <t>feature/phase7-prod-hardening</t>
-        </is>
-      </c>
-      <c r="D61" s="42" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="E61" s="42" t="inlineStr">
-        <is>
-          <t>Production hardening</t>
-        </is>
-      </c>
-      <c r="F61" s="42" t="inlineStr">
-        <is>
-          <t>Rate limiting (slowapi). Secrets management (not env file). CORS lockdown. JWT key rotation. Sentry alerts tuned for production. Load test with k6.</t>
-        </is>
-      </c>
-      <c r="G61" s="42" t="inlineStr">
-        <is>
-          <t>feat: production hardening — rate limiting, secrets, CORS, JWT rotation</t>
-        </is>
-      </c>
-      <c r="H61" s="42" t="inlineStr">
-        <is>
-          <t>docs/ROADMAP.md</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J61" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K61" s="41" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L61" s="41" t="n"/>
-      <c r="M61" s="41" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="N61" s="43" t="n">
-        <v>0</v>
-      </c>
-      <c r="O61" s="42" t="inlineStr">
-        <is>
-          <t>P7-02</t>
-        </is>
-      </c>
-      <c r="P61" s="42" t="inlineStr">
-        <is>
-          <t>Rate limit smoke test; CORS rejection; Sentry alert fires on 500; k6 load test passes</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="66" customHeight="1" s="81">
-      <c r="A62" s="22" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B62" s="22" t="inlineStr">
+      <c r="O64" t="inlineStr">
         <is>
           <t>P7-04</t>
         </is>
       </c>
-      <c r="C62" s="23" t="inlineStr">
-        <is>
-          <t>feature/phase7-docs-website</t>
-        </is>
-      </c>
-      <c r="D62" s="23" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="E62" s="23" t="inlineStr">
-        <is>
-          <t>Mintlify docs website</t>
-        </is>
-      </c>
-      <c r="F62" s="23" t="inlineStr">
-        <is>
-          <t>Point Mintlify at docs/ folder. Navigation: architecture, connectors, agents, API reference, Swiggy integration guide, evaluation, deployment. Custom domain. Public URL to share with Swiggy team, recruiters, restaurant clients.</t>
-        </is>
-      </c>
-      <c r="G62" s="23" t="inlineStr">
-        <is>
-          <t>feat: Mintlify docs website — public-facing CortexKitchen v2 documentation</t>
-        </is>
-      </c>
-      <c r="H62" s="23" t="inlineStr">
-        <is>
-          <t>All docs/ files</t>
-        </is>
-      </c>
-      <c r="I62" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J62" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K62" s="22" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L62" s="22" t="n"/>
-      <c r="M62" s="22" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="N62" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O62" s="23" t="inlineStr">
-        <is>
-          <t>P7-03</t>
-        </is>
-      </c>
-      <c r="P62" s="23" t="inlineStr">
-        <is>
-          <t>Docs site live at public URL; all 13 doc files render; search works; no broken links</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="39.6" customHeight="1" s="81">
-      <c r="A63" s="41" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B63" s="41" t="inlineStr">
-        <is>
-          <t>P7-05</t>
-        </is>
-      </c>
-      <c r="C63" s="42" t="inlineStr">
-        <is>
-          <t>dev -&gt; main PR</t>
-        </is>
-      </c>
-      <c r="D63" s="42" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="E63" s="42" t="inlineStr">
-        <is>
-          <t>Sync Phase 7 to main — public release</t>
-        </is>
-      </c>
-      <c r="F63" s="42" t="inlineStr">
-        <is>
-          <t>Live production URL. README updated with live demo link + docs website link. Apply to jobs immediately. Update portfolio.</t>
-        </is>
-      </c>
-      <c r="G63" s="42" t="inlineStr">
-        <is>
-          <t>release: Phase 7 complete — CortexKitchen v2 live in production</t>
-        </is>
-      </c>
-      <c r="H63" s="42" t="inlineStr">
-        <is>
-          <t>README.md, anoushkavyas.vercel.app portfolio</t>
-        </is>
-      </c>
-      <c r="I63" s="19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="J63" s="19" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K63" s="41" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L63" s="41" t="n"/>
-      <c r="M63" s="41" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="N63" s="43" t="n">
-        <v>0</v>
-      </c>
-      <c r="O63" s="42" t="inlineStr">
-        <is>
-          <t>P7-04</t>
-        </is>
-      </c>
-      <c r="P63" s="42" t="inlineStr">
+      <c r="P64" t="inlineStr">
         <is>
           <t>Full E2E on production URL; demo video recorded; portfolio updated</t>
         </is>

</xml_diff>

<commit_message>
tracker: mark P6-S13c Completed 2026-07-01
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -280,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -491,6 +491,7 @@
     <xf numFmtId="0" fontId="4" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13026,7 +13027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:P64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.109375" customWidth="1" style="67" min="1" max="1"/>
@@ -13138,7 +13139,8 @@
       <c r="L3" s="70" t="n"/>
       <c r="M3" s="70" t="n"/>
       <c r="N3" s="70" t="n"/>
-      <c r="O3" s="71" t="n"/>
+      <c r="O3" s="70" t="n"/>
+      <c r="P3" s="70" t="n"/>
     </row>
     <row r="4" ht="52.05" customHeight="1" s="67">
       <c r="A4" s="63" t="inlineStr">
@@ -13381,7 +13383,8 @@
       <c r="L8" s="70" t="n"/>
       <c r="M8" s="70" t="n"/>
       <c r="N8" s="70" t="n"/>
-      <c r="O8" s="71" t="n"/>
+      <c r="O8" s="70" t="n"/>
+      <c r="P8" s="70" t="n"/>
     </row>
     <row r="9" ht="52.05" customHeight="1" s="67">
       <c r="A9" s="64" t="inlineStr">
@@ -13549,7 +13552,8 @@
       <c r="L12" s="70" t="n"/>
       <c r="M12" s="70" t="n"/>
       <c r="N12" s="70" t="n"/>
-      <c r="O12" s="71" t="n"/>
+      <c r="O12" s="70" t="n"/>
+      <c r="P12" s="70" t="n"/>
     </row>
     <row r="13" ht="52.05" customHeight="1" s="67">
       <c r="A13" s="64" t="inlineStr">
@@ -14553,7 +14557,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -14566,13 +14570,18 @@
           <t>Anoushka</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>W4</t>
-        </is>
-      </c>
-      <c r="M31" t="n">
-        <v>0</v>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M31" s="78" t="n">
+        <v>1</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
tracker: Demo 1 / Demo 2 checkpoints, add P7-S06 Sarvam AI + P7-A01 AWS deployment
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -115,8 +115,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -217,6 +222,21 @@
         <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -296,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -506,6 +526,21 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -13042,7 +13077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P66"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.109375" customWidth="1" style="65" min="1" max="1"/>
@@ -14612,92 +14647,23 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="32.4" customHeight="1" s="65">
-      <c r="A32" s="78" t="inlineStr">
-        <is>
-          <t>DEMO SPRINT — build everything needed for end-to-end demo</t>
-        </is>
-      </c>
-    </row>
+    <row r="32" ht="32.4" customHeight="1" s="65"/>
     <row r="33" ht="18" customHeight="1" s="65">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>P6-F04</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-connectors</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>/connectors page — data source management</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>New route /connectors. Lists connectors with status badges (Connected/Disconnected/Error). Shows last sync time, records synced, data freshness. Connect button triggers OAuth flow. Disconnect revokes token. Error state shows last error + reconnect. Works for Swiggy + future POS connector.</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>feat: /connectors page — platform data source management with OAuth connect flow</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="M33" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>P6-S01</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>Can build now — reads from connectors table (already exists via P6-S02)</t>
+      <c r="A33" s="80" t="inlineStr">
+        <is>
+          <t>DO FIRST — no staging creds needed (connectors, market intel UI, AI upgrades, product modes)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="52.05" customHeight="1" s="65">
       <c r="A34" t="inlineStr">
         <is>
-          <t>P6-F06</t>
+          <t>P6-F04</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>feature/swiggy-frontend-market</t>
+          <t>feature/swiggy-frontend-connectors</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -14707,17 +14673,17 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Dashboard enhancements</t>
+          <t>/connectors page — data source management</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Add to existing dashboard: connector status widget (data source health bar), brief mode trigger button, today's Swiggy KPIs (orders today, delivery rating, top Swiggy seller), data_sources column on /runs list.</t>
+          <t>New route /connectors. Lists connectors with status badges (Connected/Disconnected/Error). Shows last sync time, records synced, data freshness. Connect button triggers OAuth flow. Disconnect revokes token. Error state shows last error + reconnect. Works for Swiggy + future POS connector.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>feat: dashboard — connector status widget, brief trigger, live Swiggy KPIs, data_sources on runs list</t>
+          <t>feat: /connectors page — platform data source management with OAuth connect flow</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -14755,44 +14721,44 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Can build now — connector status widget reads connectors table</t>
+          <t>Can build now — reads from connectors table (already exists via P6-S02)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="52.05" customHeight="1" s="65">
       <c r="A35" t="inlineStr">
         <is>
-          <t>P6-S14</t>
+          <t>P6-F06</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>feature/swiggy-action-queue</t>
+          <t>feature/swiggy-frontend-market</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ActionQueueService + action_queue table</t>
+          <t>Dashboard enhancements</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>New table: id, org_id, action_type (AUTO/APPROVE_REQUIRED/RECOMMENDATION), payload jsonb, status (PENDING/APPROVED/EXECUTED/REJECTED/EXPIRED), approved_by, executed_at, error. ActionQueueService CRUD. Plan output includes action_queue section in API response.</t>
+          <t>Add to existing dashboard: connector status widget (data source health bar), brief mode trigger button, today's Swiggy KPIs (orders today, delivery rating, top Swiggy seller), data_sources column on /runs list.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>feat: ActionQueueService + action_queue table — 3-tier action model with approval lifecycle</t>
+          <t>feat: dashboard — connector status widget, brief trigger, live Swiggy KPIs, data_sources on runs list</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>docs/ACTION_QUEUE.md (new), docs/APIS.md (action queue endpoints), docs/DECISIONS.md (D-021)</t>
+          <t>None (frontend only)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -14802,7 +14768,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -14812,7 +14778,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -14820,49 +14786,49 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>P6-S10</t>
+          <t>P6-S01</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>No staging creds needed — action queue is pure backend, no Swiggy write calls yet.</t>
+          <t>Can build now — connector status widget reads connectors table</t>
         </is>
       </c>
     </row>
     <row r="36" ht="52.05" customHeight="1" s="65">
       <c r="A36" t="inlineStr">
         <is>
-          <t>P6-F01</t>
+          <t>P6-S14</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>feature/swiggy-frontend-market</t>
+          <t>feature/swiggy-action-queue</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Market intelligence panel (planning results page)</t>
+          <t>ActionQueueService + action_queue table</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>New panel on /runs/{id}. Competitor pricing table: your price vs area avg vs cheapest competitor per dish category. Area occupancy badge (HIGH/MEDIUM/LOW). Instamart prices for shortage items. Pricing alerts (red if &gt;20% above area avg). Hidden when market_intel_output absent.</t>
+          <t>New table: id, org_id, action_type (AUTO/APPROVE_REQUIRED/RECOMMENDATION), payload jsonb, status (PENDING/APPROVED/EXECUTED/REJECTED/EXPIRED), approved_by, executed_at, error. ActionQueueService CRUD. Plan output includes action_queue section in API response.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>feat: market intelligence panel — competitor pricing + area occupancy on planning results</t>
+          <t>feat: ActionQueueService + action_queue table — 3-tier action model with approval lifecycle</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>None (frontend only)</t>
+          <t>docs/ACTION_QUEUE.md (new), docs/APIS.md (action queue endpoints), docs/DECISIONS.md (D-021)</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -14872,7 +14838,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -14882,7 +14848,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -14895,44 +14861,44 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Depends on P6-S11 (market_intel_output in plan API response)</t>
+          <t>No staging creds needed — action queue is pure backend, no Swiggy write calls yet.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="6" customHeight="1" s="65">
       <c r="A37" t="inlineStr">
         <is>
-          <t>P7-S04</t>
+          <t>P6-F01</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>feature/ai-upgrades</t>
+          <t>feature/swiggy-frontend-market</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Structured outputs — tool_choice=required, zero JSON hallucination</t>
+          <t>Market intelligence panel (planning results page)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Upgrade chatbot Groq calls to tool_choice=required + strict JSON schema. Apply to all 3 Swiggy chatbot tools (search_menu, get_food_orders, search_products). Chatbot function calls never hallucinate JSON. Zero model coupling — works on any provider.</t>
+          <t>New panel on /runs/{id}. Competitor pricing table: your price vs area avg vs cheapest competitor per dish category. Area occupancy badge (HIGH/MEDIUM/LOW). Instamart prices for shortage items. Pricing alerts (red if &gt;20% above area avg). Hidden when market_intel_output absent.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>feat: structured outputs — tool_choice=required across all chatbot tools</t>
+          <t>feat: market intelligence panel — competitor pricing + area occupancy on planning results</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>docs/AGENTS.md</t>
+          <t>None (frontend only)</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -14942,7 +14908,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -14952,7 +14918,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -14960,64 +14926,196 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
+          <t>P6-S10</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Depends on P6-S11 (market_intel_output in plan API response)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="65">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>P7-S04</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>feature/ai-upgrades</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Structured outputs — tool_choice=required, zero JSON hallucination</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Upgrade chatbot Groq calls to tool_choice=required + strict JSON schema. Apply to all 3 Swiggy chatbot tools (search_menu, get_food_orders, search_products). Chatbot function calls never hallucinate JSON. Zero model coupling — works on any provider.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>feat: structured outputs — tool_choice=required across all chatbot tools</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
           <t>P6-F01</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>Schema validation test; chatbot returns valid JSON on 10 consecutive calls</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1" s="65"/>
     <row r="39" ht="52.05" customHeight="1" s="65">
-      <c r="A39" s="78" t="inlineStr">
-        <is>
-          <t>RECORD END-TO-END DEMO HERE after P7-S04</t>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>P7-S01</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>feature/ai-upgrades</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Prompt caching — 60-90% cost reduction on critic + aggregator</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Add Anthropic prompt caching headers to critic and aggregator LLM calls. Both have long system prompts repeated every run. Expected saving: 60-90% of prompt token cost per planning run. Graceful fallback on cache miss. Compatible with Google Gemini too.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>feat: prompt caching — cut LLM costs 80% on critic and aggregator nodes</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>docs/ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>P7-S04</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Cost log shows cache_hit=true on second run of same scenario</t>
         </is>
       </c>
     </row>
     <row r="40" ht="52.05" customHeight="1" s="65">
-      <c r="A40" s="78" t="inlineStr">
-        <is>
-          <t>AI UPGRADES — prompt caching, reasoning model, workflow system</t>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>P7-S02</t>
         </is>
       </c>
     </row>
     <row r="41" ht="51.6" customHeight="1" s="65">
       <c r="A41" t="inlineStr">
         <is>
-          <t>P7-S01</t>
+          <t>P7-S05</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>feature/ai-upgrades</t>
+          <t>feature/workflow-system</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Prompt caching — 60-90% cost reduction on critic + aggregator</t>
+          <t>Restaurant workflow system — owner-defined trigger-condition-action automations</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Add Anthropic prompt caching headers to critic and aggregator LLM calls. Both have long system prompts repeated every run. Expected saving: 60-90% of prompt token cost per planning run. Graceful fallback on cache miss. Compatible with Google Gemini too.</t>
+          <t>New table: workflows (org_id, trigger, condition_json, action_type, action_payload, active). Triggers: AFTER_PLANNING_RUN, DAILY_BRIEF, ON_THRESHOLD. Actions: SEND_WHATSAPP, QUEUE_ACTION, CALL_WEBHOOK. WorkflowEngine evaluates conditions post-run and fires actions. /workflows UI page. Turns CortexKitchen from a tool into an OS.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>feat: prompt caching — cut LLM costs 80% on critic and aggregator nodes</t>
+          <t>feat: workflow system — restaurant owners define custom automations</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>docs/ARCHITECTURE.md</t>
+          <t>docs/ARCHITECTURE.md, docs/APIS.md</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -15037,7 +15135,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -15045,49 +15143,49 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>P7-S04</t>
+          <t>P7-S02</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Cost log shows cache_hit=true on second run of same scenario</t>
+          <t>End-to-end: planning run fires whatsapp trigger; webhook called on threshold breach</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1" s="65">
       <c r="A42" t="inlineStr">
         <is>
-          <t>P7-S02</t>
+          <t>P6-S17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>feature/ai-upgrades</t>
+          <t>feature/swiggy-brief-mode</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Reasoning model for critic — extended thinking, deeper plan evaluation</t>
+          <t>BriefingService — automated 7am daily brief</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Route critic node to Claude Opus with extended_thinking or o1/o3 via CometAPI. Critic reasons step-by-step before scoring — catches plan contradictions Sonnet misses. Falls back to Sonnet if reasoning model unavailable. One config flag: CRITIC_USE_REASONING=true. Zero coupling — model swapped via existing CometAPI registry.</t>
+          <t>APScheduler job at 07:00 IST per org. Lightweight run: demand_forecast + market_intel_node only. Pulls overnight Swiggy signals (get_food_orders since last run, track_food_order performance). Generates daily_brief JSON. Stores in daily_briefs table. Email digest (extends P5-11).</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>feat: reasoning model critic — extended thinking for deeper plan evaluation</t>
+          <t>feat: BriefingService — automated daily morning brief with overnight Swiggy signals</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>docs/AGENTS.md, docs/DECISIONS.md</t>
+          <t>docs/PRODUCT_MODES.md (new, brief mode), docs/APIS.md (brief endpoints)</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -15097,7 +15195,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -15107,7 +15205,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -15115,24 +15213,24 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>P7-S01</t>
+          <t>P6-S10</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Critic verdict quality test on 3 edge-case plans; reasoning chain logged</t>
+          <t>Scheduler fires at correct time; brief generates without full pipeline; daily_briefs row created; email sends</t>
         </is>
       </c>
     </row>
     <row r="43" ht="52.05" customHeight="1" s="65">
       <c r="A43" t="inlineStr">
         <is>
-          <t>P7-S05</t>
+          <t>P6-S18</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>feature/workflow-system</t>
+          <t>feature/swiggy-live-mode</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -15142,22 +15240,22 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Restaurant workflow system — owner-defined trigger-condition-action automations</t>
+          <t>LiveMonitorService — SSE feed during service hours</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>New table: workflows (org_id, trigger, condition_json, action_type, action_payload, active). Triggers: AFTER_PLANNING_RUN, DAILY_BRIEF, ON_THRESHOLD. Actions: SEND_WHATSAPP, QUEUE_ACTION, CALL_WEBHOOK. WorkflowEngine evaluates conditions post-run and fires actions. /workflows UI page. Turns CortexKitchen from a tool into an OS.</t>
+          <t>APScheduler-managed SSE stream active 12:00-14:00 and 19:00-22:00 IST. Polls every 30s: get_food_orders (activeOnly=true) for active delivery orders, track_food_order for in-flight ETAs, track_order for Instamart procurement status. Pushes events to /live page frontend. Alerts on: delivery &gt; SLA threshold, order spike, ingredient delivery confirmed.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>feat: workflow system — restaurant owners define custom automations</t>
+          <t>feat: LiveMonitorService — real-time Swiggy SSE during service hours (orders + procurement)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>docs/ARCHITECTURE.md, docs/APIS.md</t>
+          <t>docs/PRODUCT_MODES.md (live monitor section)</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -15167,7 +15265,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -15177,7 +15275,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -15185,56 +15283,119 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>P7-S02</t>
+          <t>P6-S17, P6-S15</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>End-to-end: planning run fires whatsapp trigger; webhook called on threshold breach</t>
+          <t>SSE stream active only during service hours IST; events emitted on each 30s poll; delivery threshold alert fires; stream stops outside service window.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="52.05" customHeight="1" s="65">
-      <c r="A44" s="79" t="inlineStr">
-        <is>
-          <t>PRODUCT COMPLETENESS — brief, live monitor, MCP, debate, voice, remaining frontend</t>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>P6-S19</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>feature/swiggy-mcp-tools</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>3 new CortexKitchen MCP server tools</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Add to mcp_server.py: get_market_brief (calls MarketIntelService live, returns competitor snapshot for Claude Desktop), get_action_queue (pending actions awaiting approval), approve_action (owner approves from Claude Desktop, triggers execution). JWT auth on all 3.</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>feat: 3 new MCP tools — get_market_brief, get_action_queue, approve_action</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>docs/APIS.md (MCP tools section), docs/ARCHITECTURE.md (MCP server updated)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>P6-S14</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>All 3 tools smoke-tested in Claude Desktop; approve_action triggers execution end-to-end; JWT enforced</t>
         </is>
       </c>
     </row>
     <row r="45" ht="52.05" customHeight="1" s="65">
       <c r="A45" t="inlineStr">
         <is>
-          <t>P6-S17</t>
+          <t>P7-S03</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>feature/swiggy-brief-mode</t>
+          <t>feature/ai-upgrades</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Agents</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>BriefingService — automated 7am daily brief</t>
+          <t>Multi-agent debate critic — two critic instances, consensus scoring</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>APScheduler job at 07:00 IST per org. Lightweight run: demand_forecast + market_intel_node only. Pulls overnight Swiggy signals (get_food_orders since last run, track_food_order performance). Generates daily_brief JSON. Stores in daily_briefs table. Email digest (extends P5-11).</t>
+          <t>Run two LLM critic instances with opposing system prompts (optimistic vs conservative). Structured debate: each scores the plan, flags disagreements, moderator LLM resolves. Final verdict is consensus or flagged-disagreement. Provably better plan quality than single critic. Zero model coupling.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>feat: BriefingService — automated daily morning brief with overnight Swiggy signals</t>
+          <t>feat: multi-agent debate critic — consensus scoring, catches more edge cases</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>docs/PRODUCT_MODES.md (new, brief mode), docs/APIS.md (brief endpoints)</t>
+          <t>docs/AGENTS.md</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -15254,7 +15415,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -15262,24 +15423,24 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>P6-S10</t>
+          <t>P7-S05</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Scheduler fires at correct time; brief generates without full pipeline; daily_briefs row created; email sends</t>
+          <t>Debate resolves on 5 test plans; disagreement cases escalate correctly</t>
         </is>
       </c>
     </row>
     <row r="46" ht="52.05" customHeight="1" s="65">
       <c r="A46" t="inlineStr">
         <is>
-          <t>P6-S18</t>
+          <t>P6-R02</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>feature/swiggy-live-mode</t>
+          <t>feature/swiggy-voice-interface</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -15289,22 +15450,22 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>LiveMonitorService — SSE feed during service hours</t>
+          <t>Voice interface — Whisper + RAG chatbot</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>APScheduler-managed SSE stream active 12:00-14:00 and 19:00-22:00 IST. Polls every 30s: get_food_orders (activeOnly=true) for active delivery orders, track_food_order for in-flight ETAs, track_order for Instamart procurement status. Pushes events to /live page frontend. Alerts on: delivery &gt; SLA threshold, order spike, ingredient delivery confirmed.</t>
+          <t>Whisper transcription on browser-recorded question (MediaRecorder API). RAG chatbot (P5-12) answers. TTS reads back. Manager asks questions while walking the floor. Works with both synthetic and real Swiggy data now in DB. Blocked on P5-12 (already done).</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>feat: LiveMonitorService — real-time Swiggy SSE during service hours (orders + procurement)</t>
+          <t>feat: voice interface — Whisper transcription + RAG answer + TTS readback</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>docs/PRODUCT_MODES.md (live monitor section)</t>
+          <t>docs/PRODUCT_MODES.md (voice section)</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -15314,7 +15475,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -15324,7 +15485,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -15332,49 +15493,49 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>P6-S17, P6-S15</t>
+          <t>P6-S16</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>SSE stream active only during service hours IST; events emitted on each 30s poll; delivery threshold alert fires; stream stops outside service window.</t>
+          <t>Transcription accuracy smoke test; end-to-end voice → RAG answer → TTS; works with real Swiggy data in DB</t>
         </is>
       </c>
     </row>
     <row r="47" ht="52.05" customHeight="1" s="65">
       <c r="A47" t="inlineStr">
         <is>
-          <t>P6-S19</t>
+          <t>P6-F02</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>feature/swiggy-mcp-tools</t>
+          <t>feature/swiggy-frontend-actions</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3 new CortexKitchen MCP server tools</t>
+          <t>Action queue UI + procurement tracker</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Add to mcp_server.py: get_market_brief (calls MarketIntelService live, returns competitor snapshot for Claude Desktop), get_action_queue (pending actions awaiting approval), approve_action (owner approves from Claude Desktop, triggers execution). JWT auth on all 3.</t>
+          <t>New section below plan output. Lists pending actions with type badge. Approve/Reject buttons for APPROVE_REQUIRED. Instamart cart preview modal (items, total, ETA) before approving checkout. Procurement tracker in inventory panel: placed orders, status, ETA.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>feat: 3 new MCP tools — get_market_brief, get_action_queue, approve_action</t>
+          <t>feat: action queue UI — approve/reject with cart preview, procurement tracker</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>docs/APIS.md (MCP tools section), docs/ARCHITECTURE.md (MCP server updated)</t>
+          <t>None (frontend only)</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -15384,7 +15545,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -15394,7 +15555,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -15402,49 +15563,49 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>P6-S14</t>
+          <t>P6-S13</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>All 3 tools smoke-tested in Claude Desktop; approve_action triggers execution end-to-end; JWT enforced</t>
+          <t>Depends on P6-S14 (action_queue in plan API response)</t>
         </is>
       </c>
     </row>
     <row r="48" ht="52.05" customHeight="1" s="65">
       <c r="A48" t="inlineStr">
         <is>
-          <t>P7-S03</t>
+          <t>P6-F03</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>feature/ai-upgrades</t>
+          <t>feature/swiggy-frontend-brief</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Multi-agent debate critic — two critic instances, consensus scoring</t>
+          <t>/brief page — daily morning briefing</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Run two LLM critic instances with opposing system prompts (optimistic vs conservative). Structured debate: each scores the plan, flags disagreements, moderator LLM resolves. Final verdict is consensus or flagged-disagreement. Provably better plan quality than single critic. Zero model coupling.</t>
+          <t>New route /brief. Overnight Swiggy performance (orders, avg delivery time, late %), today's demand forecast vs yesterday, top 3 action priorities, market snapshot. Auto-refreshes if brief is stale. Empty state when no brief yet.</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>feat: multi-agent debate critic — consensus scoring, catches more edge cases</t>
+          <t>feat: /brief page — daily morning operational briefing</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>docs/AGENTS.md</t>
+          <t>None (frontend only)</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -15464,7 +15625,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -15472,49 +15633,49 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>P7-S05</t>
+          <t>P6-S16</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Debate resolves on 5 test plans; disagreement cases escalate correctly</t>
+          <t>Depends on P6-S17 (BriefingService)</t>
         </is>
       </c>
     </row>
     <row r="49" ht="40.2" customHeight="1" s="65">
       <c r="A49" t="inlineStr">
         <is>
-          <t>P6-R02</t>
+          <t>P6-F05</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>feature/swiggy-voice-interface</t>
+          <t>feature/swiggy-frontend-live</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Voice interface — Whisper + RAG chatbot</t>
+          <t>/live page — real-time service monitor</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Whisper transcription on browser-recorded question (MediaRecorder API). RAG chatbot (P5-12) answers. TTS reads back. Manager asks questions while walking the floor. Works with both synthetic and real Swiggy data now in DB. Blocked on P5-12 (already done).</t>
+          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S18). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>feat: voice interface — Whisper transcription + RAG answer + TTS readback</t>
+          <t>feat: /live page — SSE kitchen display for active orders and procurement tracking</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>docs/PRODUCT_MODES.md (voice section)</t>
+          <t>None (frontend only)</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -15524,7 +15685,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -15542,227 +15703,26 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>P6-S16</t>
+          <t>P6-S18</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Transcription accuracy smoke test; end-to-end voice → RAG answer → TTS; works with real Swiggy data in DB</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1" s="65">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>P6-F02</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-actions</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Action queue UI + procurement tracker</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>New section below plan output. Lists pending actions with type badge. Approve/Reject buttons for APPROVE_REQUIRED. Instamart cart preview modal (items, total, ETA) before approving checkout. Procurement tracker in inventory panel: placed orders, status, ETA.</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>feat: action queue UI — approve/reject with cart preview, procurement tracker</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="M50" t="n">
-        <v>0</v>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>P6-S13</t>
-        </is>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>Depends on P6-S14 (action_queue in plan API response)</t>
-        </is>
-      </c>
-    </row>
+          <t>SSE events render in real time; ETA countdown ticks; alert banner fires on delivery spike; Swiggy branding visible; inactive state shown outside service hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1" s="65"/>
     <row r="51" ht="52.05" customHeight="1" s="65">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>P6-F03</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-brief</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>/brief page — daily morning briefing</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>New route /brief. Overnight Swiggy performance (orders, avg delivery time, late %), today's demand forecast vs yesterday, top 3 action priorities, market snapshot. Auto-refreshes if brief is stale. Empty state when no brief yet.</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>feat: /brief page — daily morning operational briefing</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="M51" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>P6-S16</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>Depends on P6-S17 (BriefingService)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="52.05" customHeight="1" s="65">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>P6-F05</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>feature/swiggy-frontend-live</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>/live page — real-time service monitor</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S18). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>feat: /live page — SSE kitchen display for active orders and procurement tracking</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="M52" t="n">
-        <v>0</v>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>P6-S18</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>SSE events render in real time; ETA countdown ticks; alert banner fires on delivery spike; Swiggy branding visible; inactive state shown outside service hours.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A51" s="81" t="inlineStr">
+        <is>
+          <t>→ DEMO 1 — record here: full Swiggy read integration + AI upgrades + voice + live monitor ←</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="52.05" customHeight="1" s="65"/>
     <row r="53" ht="52.05" customHeight="1" s="65">
-      <c r="A53" s="78" t="inlineStr">
+      <c r="A53" s="82" t="inlineStr">
         <is>
           <t>BLOCKED — needs Swiggy staging creds (write tools: checkout, book_table)</t>
         </is>
@@ -15978,117 +15938,48 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="52.05" customHeight="1" s="65">
-      <c r="A57" s="78" t="inlineStr">
-        <is>
-          <t>DOCS + PHASE 6 MILESTONE MERGE</t>
-        </is>
-      </c>
-    </row>
+    <row r="57" ht="52.05" customHeight="1" s="65"/>
     <row r="58" ht="52.05" customHeight="1" s="65">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>P6-D01</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>feature/swiggy-docs</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>5 new documentation files</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>CONNECTORS.md: BaseConnector interface, sync vs enrich, how to add new connector. SWIGGY_INTEGRATION.md: all 22 tools, parameter mappings, OAuth, rate limits, error handling. ACTION_QUEUE.md: action types, approval flow, non-idempotent patterns. DATA_SOURCES.md: all sources, channels, sync frequency. PRODUCT_MODES.md: ops/brief/live/voice mode specs.</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>docs: 5 new documentation files for Phase 6 connector + action + product mode layer</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>docs/CONNECTORS.md, docs/SWIGGY_INTEGRATION.md, docs/ACTION_QUEUE.md, docs/DATA_SOURCES.md, docs/PRODUCT_MODES.md</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="M58" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>P6-F06</t>
-        </is>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>All 5 files present; no broken links; tool parameter tables accurate vs Swiggy docs</t>
+      <c r="A58" s="83" t="inlineStr">
+        <is>
+          <t>WHEN RECEIVED — Sarvam AI access + AWS credits</t>
         </is>
       </c>
     </row>
     <row r="59" ht="52.05" customHeight="1" s="65">
       <c r="A59" t="inlineStr">
         <is>
-          <t>P6-D02</t>
+          <t>P7-S06</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>feature/swiggy-docs</t>
+          <t>feature/sarvam-voice</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Agents</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Update CLAUDE.md, README.md, Swiggy deep-dive for Phase 6 completion</t>
+          <t>Sarvam AI voice — Hindi/Hinglish speech-to-text + text-to-speech for chatbot</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>CLAUDE.md: update Current system state to Phase 6 complete (11-node pipeline, 22 Swiggy tools, full action + brief + live layer). README.md: add Phase 6 achievements, Swiggy integration summary, demo instructions. CortexKitchen_Swiggy_Deep_Dive.html: mark all chapters complete, update progress bar to 100%.</t>
+          <t>Replace Whisper plan with Sarvam ASR. Owner speaks in Hindi during service, gets response in Hindi via Sarvam TTS. Handles Hinglish and regional accents natively. Zero model coupling — Sarvam is swappable. Integrates with existing chatbot ReAct loop.</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>docs: Phase 6 milestone — CLAUDE.md, README, Swiggy deep-dive final update</t>
+          <t>feat: Sarvam AI voice — Hindi/Hinglish STT+TTS, India-native voice interface</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>CLAUDE.md, README.md, CortexKitchen_Swiggy_Deep_Dive.html</t>
+          <t>docs/AGENTS.md</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -16104,11 +15995,6 @@
       <c r="J59" t="inlineStr">
         <is>
           <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>W8</t>
         </is>
       </c>
       <c r="M59" t="n">
@@ -16116,49 +16002,49 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>P6-D01</t>
+          <t>P6-R02</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>CLAUDE.md system state accurate; README demo instructions work end-to-end; deep-dive HTML shows 100% progress.</t>
+          <t>Voice round-trip in Hindi under 3 seconds; Hinglish query understood correctly</t>
         </is>
       </c>
     </row>
     <row r="60" ht="52.05" customHeight="1" s="65">
-      <c r="A60" s="76" t="inlineStr">
-        <is>
-          <t>P6-D03</t>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>P7-A01</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>dev -&gt; main PR</t>
+          <t>feature/aws-deployment</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Phase 6 milestone merge to main</t>
+          <t>AWS production deployment — RDS, ElastiCache, ECS Fargate, GitHub Actions CI/CD</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Merge feature/ck-v2-platform → dev → main. All 11 nodes verified in LangSmith. All 22 Swiggy tools exercised in staging. POS connector imports CSV end-to-end. Voice interface smoke tested. Action queue end-to-end. All 3 product modes verified. 5 new frontend pages smoke tested. Full test suite green.</t>
+          <t>PostgreSQL → RDS, Redis → ElastiCache, API → ECS Fargate (containerised), frontend → Vercel/Amplify, exports → S3. GitHub Actions pipeline: test → build → push ECR → deploy ECS. SSL cert. One-command deploy. Uses AWS credits. Zero downtime deploys.</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>release: Phase 6 complete — CortexKitchen v2 Swiggy-native restaurant OS</t>
+          <t>feat: AWS production deployment — containerised, auto-scaling, CI/CD pipeline</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>README.md (portfolio headline), docs/ROADMAP.md (Phase 6 complete)</t>
+          <t>docs/ARCHITECTURE.md</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -16168,17 +16054,12 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
           <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>W8</t>
         </is>
       </c>
       <c r="M60" t="n">
@@ -16186,241 +16067,40 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>P6-D02</t>
+          <t>P7-01</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Full test suite green; 11 nodes in LangSmith; staging demo clean; portfolio README updated; docs website prep checklist done</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="38.4" customHeight="1" s="65">
-      <c r="A61" s="78" t="inlineStr">
-        <is>
-          <t>PHASE 7 — Production, CI/CD, Public Release</t>
-        </is>
-      </c>
-    </row>
+          <t>Full deploy from scratch via one make command; zero-downtime redeploy verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="38.4" customHeight="1" s="65"/>
     <row r="62" ht="66" customHeight="1" s="65">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>P7-01</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>feature/phase7-cicd</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>CI/CD — GitHub Actions</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Automated on every PR: unit + integration + RAGAS evals + DeepEval; lint; type check; frontend build; coverage report. Fail on critic score regression. Cache pip dependencies.</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>feat: CI/CD — automated test + eval pipeline on every PR</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>docs/ROADMAP.md</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="M62" t="n">
-        <v>0</v>
-      </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>P6-D03</t>
-        </is>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>CI passes on clean repo; fails on intentional test break; eval regression detected</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="39.6" customHeight="1" s="65">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>P7-02</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>feature/phase7-cloud-deploy</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Cloud deployment — Railway / Fly.io</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Containerise API + frontend. Deploy to Railway or Fly.io. Managed Postgres + Redis + Qdrant. Production env vars. Swiggy OAuth redirect URI updated for production domain. Health endpoint green on production URL.</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>feat: cloud deployment — production on Railway/Fly.io</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>docs/ROADMAP.md</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="M63" t="n">
-        <v>0</v>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>P7-01</t>
-        </is>
-      </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t>Production URL health check green; all env vars; Swiggy OAuth works on production domain</t>
-        </is>
-      </c>
-    </row>
+      <c r="A62" s="81" t="inlineStr">
+        <is>
+          <t>→ DEMO 2 / POTENTIAL DEMO — full product: write tools + Sarvam voice + AWS hosted ←</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="39.6" customHeight="1" s="65"/>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>P7-03</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>feature/phase7-prod-hardening</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Production hardening</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Rate limiting (slowapi). Secrets management (not env file). CORS lockdown. JWT key rotation. Sentry alerts tuned for production. Load test with k6.</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>feat: production hardening — rate limiting, secrets, CORS, JWT rotation</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>docs/ROADMAP.md</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="M64" t="n">
-        <v>0</v>
-      </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>P7-02</t>
-        </is>
-      </c>
-      <c r="O64" t="inlineStr">
-        <is>
-          <t>Rate limit smoke test; CORS rejection; Sentry alert fires on 500; k6 load test passes</t>
+      <c r="A64" s="84" t="inlineStr">
+        <is>
+          <t>DOCS + PHASE 6 MILESTONE MERGE</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>P7-04</t>
+          <t>P6-D01</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>feature/phase7-docs-website</t>
+          <t>feature/swiggy-docs</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -16430,22 +16110,22 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mintlify docs website</t>
+          <t>5 new documentation files</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Point Mintlify at docs/ folder. Navigation: architecture, connectors, agents, API reference, Swiggy integration guide, evaluation, deployment. Custom domain. Public URL to share with Swiggy team, recruiters, restaurant clients.</t>
+          <t>CONNECTORS.md: BaseConnector interface, sync vs enrich, how to add new connector. SWIGGY_INTEGRATION.md: all 22 tools, parameter mappings, OAuth, rate limits, error handling. ACTION_QUEUE.md: action types, approval flow, non-idempotent patterns. DATA_SOURCES.md: all sources, channels, sync frequency. PRODUCT_MODES.md: ops/brief/live/voice mode specs.</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>feat: Mintlify docs website — public-facing CortexKitchen v2 documentation</t>
+          <t>docs: 5 new documentation files for Phase 6 connector + action + product mode layer</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>All docs/ files</t>
+          <t>docs/CONNECTORS.md, docs/SWIGGY_INTEGRATION.md, docs/ACTION_QUEUE.md, docs/DATA_SOURCES.md, docs/PRODUCT_MODES.md</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -16455,7 +16135,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -16465,7 +16145,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="M65" t="n">
@@ -16473,49 +16153,49 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>P7-03</t>
+          <t>P6-F06</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Docs site live at public URL; all 13 doc files render; search works; no broken links</t>
+          <t>All 5 files present; no broken links; tool parameter tables accurate vs Swiggy docs</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>P7-05</t>
+          <t>P6-D02</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>dev -&gt; main PR</t>
+          <t>feature/swiggy-docs</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Sync Phase 7 to main — public release</t>
+          <t>Update CLAUDE.md, README.md, Swiggy deep-dive for Phase 6 completion</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Live production URL. README updated with live demo link + docs website link. Apply to jobs immediately. Update portfolio.</t>
+          <t>CLAUDE.md: update Current system state to Phase 6 complete (11-node pipeline, 22 Swiggy tools, full action + brief + live layer). README.md: add Phase 6 achievements, Swiggy integration summary, demo instructions. CortexKitchen_Swiggy_Deep_Dive.html: mark all chapters complete, update progress bar to 100%.</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>release: Phase 7 complete — CortexKitchen v2 live in production</t>
+          <t>docs: Phase 6 milestone — CLAUDE.md, README, Swiggy deep-dive final update</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>README.md, anoushkavyas.vercel.app portfolio</t>
+          <t>CLAUDE.md, README.md, CortexKitchen_Swiggy_Deep_Dive.html</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -16525,7 +16205,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -16535,7 +16215,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="M66" t="n">
@@ -16543,10 +16223,438 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
+          <t>P6-D01</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>CLAUDE.md system state accurate; README demo instructions work end-to-end; deep-dive HTML shows 100% progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>P6-D03</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>dev -&gt; main PR</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Phase 6 milestone merge to main</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Merge feature/ck-v2-platform → dev → main. All 11 nodes verified in LangSmith. All 22 Swiggy tools exercised in staging. POS connector imports CSV end-to-end. Voice interface smoke tested. Action queue end-to-end. All 3 product modes verified. 5 new frontend pages smoke tested. Full test suite green.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>release: Phase 6 complete — CortexKitchen v2 Swiggy-native restaurant OS</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>README.md (portfolio headline), docs/ROADMAP.md (Phase 6 complete)</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>P6-D02</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Full test suite green; 11 nodes in LangSmith; staging demo clean; portfolio README updated; docs website prep checklist done</t>
+        </is>
+      </c>
+    </row>
+    <row r="68"/>
+    <row r="69">
+      <c r="A69" s="84" t="inlineStr">
+        <is>
+          <t>PHASE 7 — Production, CI/CD, Public Release</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>P7-01</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>feature/phase7-cicd</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>CI/CD — GitHub Actions</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Automated on every PR: unit + integration + RAGAS evals + DeepEval; lint; type check; frontend build; coverage report. Fail on critic score regression. Cache pip dependencies.</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>feat: CI/CD — automated test + eval pipeline on every PR</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>docs/ROADMAP.md</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>P6-D03</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>CI passes on clean repo; fails on intentional test break; eval regression detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>P7-02</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>feature/phase7-cloud-deploy</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Cloud deployment — Railway / Fly.io</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Containerise API + frontend. Deploy to Railway or Fly.io. Managed Postgres + Redis + Qdrant. Production env vars. Swiggy OAuth redirect URI updated for production domain. Health endpoint green on production URL.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>feat: cloud deployment — production on Railway/Fly.io</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>docs/ROADMAP.md</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>P7-01</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Production URL health check green; all env vars; Swiggy OAuth works on production domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>P7-03</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>feature/phase7-prod-hardening</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Production hardening</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Rate limiting (slowapi). Secrets management (not env file). CORS lockdown. JWT key rotation. Sentry alerts tuned for production. Load test with k6.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>feat: production hardening — rate limiting, secrets, CORS, JWT rotation</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>docs/ROADMAP.md</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>P7-02</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Rate limit smoke test; CORS rejection; Sentry alert fires on 500; k6 load test passes</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>P7-04</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>feature/phase7-docs-website</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Mintlify docs website</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Point Mintlify at docs/ folder. Navigation: architecture, connectors, agents, API reference, Swiggy integration guide, evaluation, deployment. Custom domain. Public URL to share with Swiggy team, recruiters, restaurant clients.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>feat: Mintlify docs website — public-facing CortexKitchen v2 documentation</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>All docs/ files</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="M73" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>P7-03</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Docs site live at public URL; all 13 doc files render; search works; no broken links</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>P7-05</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>dev -&gt; main PR</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Sync Phase 7 to main — public release</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Live production URL. README updated with live demo link + docs website link. Apply to jobs immediately. Update portfolio.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>release: Phase 7 complete — CortexKitchen v2 live in production</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>README.md, anoushkavyas.vercel.app portfolio</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="M74" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>P7-04</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
         <is>
           <t>Full E2E on production URL; demo video recorded; portfolio updated</t>
         </is>

</xml_diff>

<commit_message>
tracker: clean P7 IDs — P7-01 through P7-13, no letter suffixes
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -14965,7 +14965,7 @@
     <row r="36" ht="40.05" customHeight="1" s="82">
       <c r="A36" s="87" t="inlineStr">
         <is>
-          <t>P7-S01</t>
+          <t>P7-01</t>
         </is>
       </c>
       <c r="B36" s="87" t="inlineStr">
@@ -15035,7 +15035,7 @@
     <row r="37" ht="40.05" customHeight="1" s="82">
       <c r="A37" s="87" t="inlineStr">
         <is>
-          <t>P7-S02</t>
+          <t>P7-02</t>
         </is>
       </c>
       <c r="B37" s="87" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="N37" s="87" t="inlineStr">
         <is>
-          <t>P7-S01</t>
+          <t>P7-01</t>
         </is>
       </c>
       <c r="O37" s="87" t="inlineStr">
@@ -15105,14 +15105,14 @@
     <row r="38" ht="40.05" customHeight="1" s="82">
       <c r="A38" s="87" t="inlineStr">
         <is>
-          <t>P7-S03</t>
+          <t>P7-03</t>
         </is>
       </c>
     </row>
     <row r="39" ht="40.05" customHeight="1" s="82">
       <c r="A39" s="87" t="inlineStr">
         <is>
-          <t>P7-S04</t>
+          <t>P7-04</t>
         </is>
       </c>
       <c r="B39" s="87" t="inlineStr">
@@ -15170,7 +15170,7 @@
       </c>
       <c r="N39" s="87" t="inlineStr">
         <is>
-          <t>P7-S03</t>
+          <t>P7-03</t>
         </is>
       </c>
       <c r="O39" s="87" t="inlineStr">
@@ -15329,7 +15329,7 @@
     <row r="43" ht="40.05" customHeight="1" s="82">
       <c r="A43" s="87" t="inlineStr">
         <is>
-          <t>P7-S05</t>
+          <t>P7-05</t>
         </is>
       </c>
       <c r="B43" s="87" t="inlineStr">
@@ -15387,7 +15387,7 @@
       </c>
       <c r="N43" s="87" t="inlineStr">
         <is>
-          <t>P7-S04</t>
+          <t>P7-04</t>
         </is>
       </c>
       <c r="O43" s="87" t="inlineStr">
@@ -15835,7 +15835,7 @@
     <row r="54" ht="40.05" customHeight="1" s="82">
       <c r="A54" s="87" t="inlineStr">
         <is>
-          <t>P7-S07</t>
+          <t>P7-07</t>
         </is>
       </c>
       <c r="B54" s="87" t="inlineStr">
@@ -15893,7 +15893,7 @@
       </c>
       <c r="N54" s="87" t="inlineStr">
         <is>
-          <t>P7-S05</t>
+          <t>P7-05</t>
         </is>
       </c>
       <c r="O54" s="87" t="inlineStr">
@@ -15913,7 +15913,7 @@
     <row r="57" ht="40.05" customHeight="1" s="82">
       <c r="A57" s="87" t="inlineStr">
         <is>
-          <t>P7-S06</t>
+          <t>P7-06</t>
         </is>
       </c>
       <c r="B57" s="87" t="inlineStr">
@@ -15978,7 +15978,7 @@
     <row r="58" ht="40.05" customHeight="1" s="82">
       <c r="A58" s="87" t="inlineStr">
         <is>
-          <t>P7-I01</t>
+          <t>P7-08</t>
         </is>
       </c>
       <c r="B58" s="87" t="inlineStr">
@@ -16031,7 +16031,7 @@
       </c>
       <c r="N58" s="87" t="inlineStr">
         <is>
-          <t>P7-P01</t>
+          <t>P7-09</t>
         </is>
       </c>
       <c r="O58" s="87" t="inlineStr">
@@ -16277,7 +16277,7 @@
     <row r="68" ht="40.05" customHeight="1" s="82">
       <c r="A68" s="87" t="inlineStr">
         <is>
-          <t>P7-P01</t>
+          <t>P7-09</t>
         </is>
       </c>
       <c r="B68" s="87" t="inlineStr">
@@ -16347,7 +16347,7 @@
     <row r="69" ht="40.05" customHeight="1" s="82">
       <c r="A69" s="87" t="inlineStr">
         <is>
-          <t>P7-P02</t>
+          <t>P7-10</t>
         </is>
       </c>
       <c r="B69" s="87" t="inlineStr">
@@ -16405,7 +16405,7 @@
       </c>
       <c r="N69" s="87" t="inlineStr">
         <is>
-          <t>P7-P01</t>
+          <t>P7-09</t>
         </is>
       </c>
       <c r="O69" s="87" t="inlineStr">
@@ -16417,7 +16417,7 @@
     <row r="70" ht="40.05" customHeight="1" s="82">
       <c r="A70" s="87" t="inlineStr">
         <is>
-          <t>P7-P03</t>
+          <t>P7-11</t>
         </is>
       </c>
       <c r="B70" s="87" t="inlineStr">
@@ -16475,7 +16475,7 @@
       </c>
       <c r="N70" s="87" t="inlineStr">
         <is>
-          <t>P7-P02</t>
+          <t>P7-10</t>
         </is>
       </c>
       <c r="O70" s="87" t="inlineStr">
@@ -16487,7 +16487,7 @@
     <row r="71" ht="40.05" customHeight="1" s="82">
       <c r="A71" s="87" t="inlineStr">
         <is>
-          <t>P7-P04</t>
+          <t>P7-12</t>
         </is>
       </c>
       <c r="B71" s="87" t="inlineStr">
@@ -16545,7 +16545,7 @@
       </c>
       <c r="N71" s="87" t="inlineStr">
         <is>
-          <t>P7-P03</t>
+          <t>P7-11</t>
         </is>
       </c>
       <c r="O71" s="87" t="inlineStr">
@@ -16557,7 +16557,7 @@
     <row r="72" ht="40.05" customHeight="1" s="82">
       <c r="A72" s="87" t="inlineStr">
         <is>
-          <t>P7-P05</t>
+          <t>P7-13</t>
         </is>
       </c>
       <c r="B72" s="87" t="inlineStr">
@@ -16615,7 +16615,7 @@
       </c>
       <c r="N72" s="87" t="inlineStr">
         <is>
-          <t>P7-P04</t>
+          <t>P7-12</t>
         </is>
       </c>
       <c r="O72" s="87" t="inlineStr">
@@ -17001,7 +17001,7 @@
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>P7-P04 — Phase 7</t>
+          <t>P7-12 — Phase 7</t>
         </is>
       </c>
       <c r="D17" s="27" t="inlineStr">

</xml_diff>

<commit_message>
tracker: fix phases — P6-S20..S27 for AI/feature tasks, P7 = production only (P7-01..05)
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -14965,7 +14965,7 @@
     <row r="36" ht="40.05" customHeight="1" s="82">
       <c r="A36" s="87" t="inlineStr">
         <is>
-          <t>P7-01</t>
+          <t>P6-S20</t>
         </is>
       </c>
       <c r="B36" s="87" t="inlineStr">
@@ -15035,7 +15035,7 @@
     <row r="37" ht="40.05" customHeight="1" s="82">
       <c r="A37" s="87" t="inlineStr">
         <is>
-          <t>P7-02</t>
+          <t>P6-S21</t>
         </is>
       </c>
       <c r="B37" s="87" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="N37" s="87" t="inlineStr">
         <is>
-          <t>P7-01</t>
+          <t>P6-S20</t>
         </is>
       </c>
       <c r="O37" s="87" t="inlineStr">
@@ -15105,14 +15105,14 @@
     <row r="38" ht="40.05" customHeight="1" s="82">
       <c r="A38" s="87" t="inlineStr">
         <is>
-          <t>P7-03</t>
+          <t>P6-S22</t>
         </is>
       </c>
     </row>
     <row r="39" ht="40.05" customHeight="1" s="82">
       <c r="A39" s="87" t="inlineStr">
         <is>
-          <t>P7-04</t>
+          <t>P6-S23</t>
         </is>
       </c>
       <c r="B39" s="87" t="inlineStr">
@@ -15170,7 +15170,7 @@
       </c>
       <c r="N39" s="87" t="inlineStr">
         <is>
-          <t>P7-03</t>
+          <t>P6-S22</t>
         </is>
       </c>
       <c r="O39" s="87" t="inlineStr">
@@ -15329,7 +15329,7 @@
     <row r="43" ht="40.05" customHeight="1" s="82">
       <c r="A43" s="87" t="inlineStr">
         <is>
-          <t>P7-05</t>
+          <t>P6-S24</t>
         </is>
       </c>
       <c r="B43" s="87" t="inlineStr">
@@ -15387,7 +15387,7 @@
       </c>
       <c r="N43" s="87" t="inlineStr">
         <is>
-          <t>P7-04</t>
+          <t>P6-S23</t>
         </is>
       </c>
       <c r="O43" s="87" t="inlineStr">
@@ -15835,7 +15835,7 @@
     <row r="54" ht="40.05" customHeight="1" s="82">
       <c r="A54" s="87" t="inlineStr">
         <is>
-          <t>P7-07</t>
+          <t>P6-S26</t>
         </is>
       </c>
       <c r="B54" s="87" t="inlineStr">
@@ -15893,7 +15893,7 @@
       </c>
       <c r="N54" s="87" t="inlineStr">
         <is>
-          <t>P7-05</t>
+          <t>P6-S24</t>
         </is>
       </c>
       <c r="O54" s="87" t="inlineStr">
@@ -15913,7 +15913,7 @@
     <row r="57" ht="40.05" customHeight="1" s="82">
       <c r="A57" s="87" t="inlineStr">
         <is>
-          <t>P7-06</t>
+          <t>P6-S25</t>
         </is>
       </c>
       <c r="B57" s="87" t="inlineStr">
@@ -15978,7 +15978,7 @@
     <row r="58" ht="40.05" customHeight="1" s="82">
       <c r="A58" s="87" t="inlineStr">
         <is>
-          <t>P7-08</t>
+          <t>P6-S27</t>
         </is>
       </c>
       <c r="B58" s="87" t="inlineStr">
@@ -16031,7 +16031,7 @@
       </c>
       <c r="N58" s="87" t="inlineStr">
         <is>
-          <t>P7-09</t>
+          <t>P7-01</t>
         </is>
       </c>
       <c r="O58" s="87" t="inlineStr">
@@ -16277,7 +16277,7 @@
     <row r="68" ht="40.05" customHeight="1" s="82">
       <c r="A68" s="87" t="inlineStr">
         <is>
-          <t>P7-09</t>
+          <t>P7-01</t>
         </is>
       </c>
       <c r="B68" s="87" t="inlineStr">
@@ -16347,7 +16347,7 @@
     <row r="69" ht="40.05" customHeight="1" s="82">
       <c r="A69" s="87" t="inlineStr">
         <is>
-          <t>P7-10</t>
+          <t>P7-02</t>
         </is>
       </c>
       <c r="B69" s="87" t="inlineStr">
@@ -16405,7 +16405,7 @@
       </c>
       <c r="N69" s="87" t="inlineStr">
         <is>
-          <t>P7-09</t>
+          <t>P7-01</t>
         </is>
       </c>
       <c r="O69" s="87" t="inlineStr">
@@ -16417,7 +16417,7 @@
     <row r="70" ht="40.05" customHeight="1" s="82">
       <c r="A70" s="87" t="inlineStr">
         <is>
-          <t>P7-11</t>
+          <t>P7-03</t>
         </is>
       </c>
       <c r="B70" s="87" t="inlineStr">
@@ -16475,7 +16475,7 @@
       </c>
       <c r="N70" s="87" t="inlineStr">
         <is>
-          <t>P7-10</t>
+          <t>P7-02</t>
         </is>
       </c>
       <c r="O70" s="87" t="inlineStr">
@@ -16487,7 +16487,7 @@
     <row r="71" ht="40.05" customHeight="1" s="82">
       <c r="A71" s="87" t="inlineStr">
         <is>
-          <t>P7-12</t>
+          <t>P7-04</t>
         </is>
       </c>
       <c r="B71" s="87" t="inlineStr">
@@ -16545,7 +16545,7 @@
       </c>
       <c r="N71" s="87" t="inlineStr">
         <is>
-          <t>P7-11</t>
+          <t>P7-03</t>
         </is>
       </c>
       <c r="O71" s="87" t="inlineStr">
@@ -16557,7 +16557,7 @@
     <row r="72" ht="40.05" customHeight="1" s="82">
       <c r="A72" s="87" t="inlineStr">
         <is>
-          <t>P7-13</t>
+          <t>P7-05</t>
         </is>
       </c>
       <c r="B72" s="87" t="inlineStr">
@@ -16615,7 +16615,7 @@
       </c>
       <c r="N72" s="87" t="inlineStr">
         <is>
-          <t>P7-12</t>
+          <t>P7-04</t>
         </is>
       </c>
       <c r="O72" s="87" t="inlineStr">
@@ -17001,7 +17001,7 @@
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>P7-12 — Phase 7</t>
+          <t>P7-04 — Phase 7</t>
         </is>
       </c>
       <c r="D17" s="27" t="inlineStr">

</xml_diff>

<commit_message>
tracker: final renumber — task number = sequential position in P6 (F14..F29, S16..S34, R26, D35..D37)
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v5.xlsx
+++ b/CortexKitchen_Progress_Tracker_v5.xlsx
@@ -1023,7 +1023,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Pending from Swiggy. Needed ONLY for checkout + book_table (P6-S15, P6-S16). Everything else works with production OAuth token.</t>
+          <t>Pending from Swiggy. Needed ONLY for checkout + book_table (P6-S30, P6-S31). Everything else works with production OAuth token.</t>
         </is>
       </c>
       <c r="C6" s="1" t="n"/>
@@ -13951,12 +13951,12 @@
       </c>
       <c r="E16" s="87" t="inlineStr">
         <is>
-          <t>Create sync/reservation_sync.py. sync() calls get_booking_status per registered Dineout orderId. Graceful no-op until book_table (P6-S16) registers booking IDs. register_booking_order_id() stores Dineout order IDs in connector_metadata JSONB. Dedup by external_booking_id. source=dineout. Migration d2c8f1e4b7a9 adds connectors.connector_metadata + feedback.external_order_id.</t>
+          <t>Create sync/reservation_sync.py. sync() calls get_booking_status per registered Dineout orderId. Graceful no-op until book_table (P6-S31) registers booking IDs. register_booking_order_id() stores Dineout order IDs in connector_metadata JSONB. Dedup by external_booking_id. source=dineout. Migration d2c8f1e4b7a9 adds connectors.connector_metadata + feedback.external_order_id.</t>
         </is>
       </c>
       <c r="F16" s="87" t="inlineStr">
         <is>
-          <t>feat: reservation sync skeleton — get_booking_status → reservations table, register_booking_order_id for DineoutExecutor (P6-S16)</t>
+          <t>feat: reservation sync skeleton — get_booking_status → reservations table, register_booking_order_id for DineoutExecutor (P6-S31)</t>
         </is>
       </c>
       <c r="G16" s="87" t="inlineStr">
@@ -14251,7 +14251,7 @@
       </c>
       <c r="E22" s="21" t="inlineStr">
         <is>
-          <t>Create enrichers/procurement.py. search_products (per shortage item, max 5 calls/run) + your_go_to_items (frequent reorders). Output: [{ingredient, spinId, price, unit, inStock}]. spinId MUST persist in OrchestratorState — required for Instamart checkout in P6-S15. Redis cache 30 min. Returns None on any failure; inventory node falls back to its own analysis.</t>
+          <t>Create enrichers/procurement.py. search_products (per shortage item, max 5 calls/run) + your_go_to_items (frequent reorders). Output: [{ingredient, spinId, price, unit, inStock}]. spinId MUST persist in OrchestratorState — required for Instamart checkout in P6-S30. Redis cache 30 min. Returns None on any failure; inventory node falls back to its own analysis.</t>
         </is>
       </c>
       <c r="F22" s="21" t="inlineStr">
@@ -14685,7 +14685,7 @@
     <row r="32" ht="40.05" customHeight="1" s="82">
       <c r="A32" s="87" t="inlineStr">
         <is>
-          <t>P6-F04</t>
+          <t>P6-F14</t>
         </is>
       </c>
       <c r="B32" s="87" t="inlineStr">
@@ -14755,7 +14755,7 @@
     <row r="33" ht="40.05" customHeight="1" s="82">
       <c r="A33" s="87" t="inlineStr">
         <is>
-          <t>P6-F06</t>
+          <t>P6-F15</t>
         </is>
       </c>
       <c r="B33" s="87" t="inlineStr">
@@ -14825,7 +14825,7 @@
     <row r="34" ht="40.05" customHeight="1" s="82">
       <c r="A34" s="87" t="inlineStr">
         <is>
-          <t>P6-S14</t>
+          <t>P6-S16</t>
         </is>
       </c>
       <c r="B34" s="87" t="inlineStr">
@@ -14895,7 +14895,7 @@
     <row r="35" ht="40.05" customHeight="1" s="82">
       <c r="A35" s="87" t="inlineStr">
         <is>
-          <t>P6-F01</t>
+          <t>P6-F17</t>
         </is>
       </c>
       <c r="B35" s="87" t="inlineStr">
@@ -14965,7 +14965,7 @@
     <row r="36" ht="40.05" customHeight="1" s="82">
       <c r="A36" s="87" t="inlineStr">
         <is>
-          <t>P6-S20</t>
+          <t>P6-S18</t>
         </is>
       </c>
       <c r="B36" s="87" t="inlineStr">
@@ -15023,7 +15023,7 @@
       </c>
       <c r="N36" s="87" t="inlineStr">
         <is>
-          <t>P6-F01</t>
+          <t>P6-F17</t>
         </is>
       </c>
       <c r="O36" s="87" t="inlineStr">
@@ -15035,7 +15035,7 @@
     <row r="37" ht="40.05" customHeight="1" s="82">
       <c r="A37" s="87" t="inlineStr">
         <is>
-          <t>P6-S21</t>
+          <t>P6-S19</t>
         </is>
       </c>
       <c r="B37" s="87" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="N37" s="87" t="inlineStr">
         <is>
-          <t>P6-S20</t>
+          <t>P6-S18</t>
         </is>
       </c>
       <c r="O37" s="87" t="inlineStr">
@@ -15105,14 +15105,14 @@
     <row r="38" ht="40.05" customHeight="1" s="82">
       <c r="A38" s="87" t="inlineStr">
         <is>
-          <t>P6-S22</t>
+          <t>P6-S20</t>
         </is>
       </c>
     </row>
     <row r="39" ht="40.05" customHeight="1" s="82">
       <c r="A39" s="87" t="inlineStr">
         <is>
-          <t>P6-S23</t>
+          <t>P6-S21</t>
         </is>
       </c>
       <c r="B39" s="87" t="inlineStr">
@@ -15170,7 +15170,7 @@
       </c>
       <c r="N39" s="87" t="inlineStr">
         <is>
-          <t>P6-S22</t>
+          <t>P6-S20</t>
         </is>
       </c>
       <c r="O39" s="87" t="inlineStr">
@@ -15182,14 +15182,14 @@
     <row r="40" ht="40.05" customHeight="1" s="82">
       <c r="A40" s="86" t="inlineStr">
         <is>
-          <t>P6-S17</t>
+          <t>P6-S22</t>
         </is>
       </c>
     </row>
     <row r="41" ht="40.05" customHeight="1" s="82">
       <c r="A41" s="87" t="inlineStr">
         <is>
-          <t>P6-S18</t>
+          <t>P6-S23</t>
         </is>
       </c>
       <c r="B41" s="87" t="inlineStr">
@@ -15247,7 +15247,7 @@
       </c>
       <c r="N41" s="87" t="inlineStr">
         <is>
-          <t>P6-S17, P6-S15</t>
+          <t>P6-S22, P6-S30</t>
         </is>
       </c>
       <c r="O41" s="87" t="inlineStr">
@@ -15259,7 +15259,7 @@
     <row r="42" ht="40.05" customHeight="1" s="82">
       <c r="A42" s="87" t="inlineStr">
         <is>
-          <t>P6-S19</t>
+          <t>P6-S24</t>
         </is>
       </c>
       <c r="B42" s="87" t="inlineStr">
@@ -15317,7 +15317,7 @@
       </c>
       <c r="N42" s="87" t="inlineStr">
         <is>
-          <t>P6-S14</t>
+          <t>P6-S16</t>
         </is>
       </c>
       <c r="O42" s="87" t="inlineStr">
@@ -15329,7 +15329,7 @@
     <row r="43" ht="40.05" customHeight="1" s="82">
       <c r="A43" s="87" t="inlineStr">
         <is>
-          <t>P6-S24</t>
+          <t>P6-S25</t>
         </is>
       </c>
       <c r="B43" s="87" t="inlineStr">
@@ -15387,7 +15387,7 @@
       </c>
       <c r="N43" s="87" t="inlineStr">
         <is>
-          <t>P6-S23</t>
+          <t>P6-S21</t>
         </is>
       </c>
       <c r="O43" s="87" t="inlineStr">
@@ -15399,7 +15399,7 @@
     <row r="44" ht="40.05" customHeight="1" s="82">
       <c r="A44" s="87" t="inlineStr">
         <is>
-          <t>P6-R02</t>
+          <t>P6-R26</t>
         </is>
       </c>
       <c r="B44" s="87" t="inlineStr">
@@ -15457,7 +15457,7 @@
       </c>
       <c r="N44" s="87" t="inlineStr">
         <is>
-          <t>P6-S16</t>
+          <t>P6-S31</t>
         </is>
       </c>
       <c r="O44" s="87" t="inlineStr">
@@ -15469,7 +15469,7 @@
     <row r="45" ht="40.05" customHeight="1" s="82">
       <c r="A45" s="87" t="inlineStr">
         <is>
-          <t>P6-F02</t>
+          <t>P6-F27</t>
         </is>
       </c>
       <c r="B45" s="87" t="inlineStr">
@@ -15532,14 +15532,14 @@
       </c>
       <c r="O45" s="87" t="inlineStr">
         <is>
-          <t>Depends on P6-S14 (action_queue in plan API response)</t>
+          <t>Depends on P6-S16 (action_queue in plan API response)</t>
         </is>
       </c>
     </row>
     <row r="46" ht="40.05" customHeight="1" s="82">
       <c r="A46" s="87" t="inlineStr">
         <is>
-          <t>P6-F03</t>
+          <t>P6-F28</t>
         </is>
       </c>
       <c r="B46" s="87" t="inlineStr">
@@ -15597,19 +15597,19 @@
       </c>
       <c r="N46" s="87" t="inlineStr">
         <is>
-          <t>P6-S16</t>
+          <t>P6-S31</t>
         </is>
       </c>
       <c r="O46" s="87" t="inlineStr">
         <is>
-          <t>Depends on P6-S17 (BriefingService)</t>
+          <t>Depends on P6-S22 (BriefingService)</t>
         </is>
       </c>
     </row>
     <row r="47" ht="40.05" customHeight="1" s="82">
       <c r="A47" s="87" t="inlineStr">
         <is>
-          <t>P6-F05</t>
+          <t>P6-F29</t>
         </is>
       </c>
       <c r="B47" s="87" t="inlineStr">
@@ -15629,7 +15629,7 @@
       </c>
       <c r="E47" s="87" t="inlineStr">
         <is>
-          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S18). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
+          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S23). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
         </is>
       </c>
       <c r="F47" s="87" t="inlineStr">
@@ -15667,7 +15667,7 @@
       </c>
       <c r="N47" s="87" t="inlineStr">
         <is>
-          <t>P6-S18</t>
+          <t>P6-S23</t>
         </is>
       </c>
       <c r="O47" s="87" t="inlineStr">
@@ -15695,7 +15695,7 @@
     <row r="52" ht="40.05" customHeight="1" s="82">
       <c r="A52" s="87" t="inlineStr">
         <is>
-          <t>P6-S15</t>
+          <t>P6-S30</t>
         </is>
       </c>
       <c r="B52" s="87" t="inlineStr">
@@ -15725,7 +15725,7 @@
       </c>
       <c r="G52" s="87" t="inlineStr">
         <is>
-          <t>docs/SWIGGY_INTEGRATION.md (P6-S15 executor section)</t>
+          <t>docs/SWIGGY_INTEGRATION.md (P6-S30 executor section)</t>
         </is>
       </c>
       <c r="H52" s="87" t="inlineStr">
@@ -15753,7 +15753,7 @@
       </c>
       <c r="N52" s="87" t="inlineStr">
         <is>
-          <t>P6-S14, P6-S09</t>
+          <t>P6-S16, P6-S09</t>
         </is>
       </c>
       <c r="O52" s="87" t="inlineStr">
@@ -15765,7 +15765,7 @@
     <row r="53" ht="40.05" customHeight="1" s="82">
       <c r="A53" s="87" t="inlineStr">
         <is>
-          <t>P6-S16</t>
+          <t>P6-S31</t>
         </is>
       </c>
       <c r="B53" s="87" t="inlineStr">
@@ -15823,7 +15823,7 @@
       </c>
       <c r="N53" s="87" t="inlineStr">
         <is>
-          <t>P6-S14</t>
+          <t>P6-S16</t>
         </is>
       </c>
       <c r="O53" s="87" t="inlineStr">
@@ -15835,7 +15835,7 @@
     <row r="54" ht="40.05" customHeight="1" s="82">
       <c r="A54" s="87" t="inlineStr">
         <is>
-          <t>P6-S26</t>
+          <t>P6-S32</t>
         </is>
       </c>
       <c r="B54" s="87" t="inlineStr">
@@ -15893,7 +15893,7 @@
       </c>
       <c r="N54" s="87" t="inlineStr">
         <is>
-          <t>P6-S24</t>
+          <t>P6-S25</t>
         </is>
       </c>
       <c r="O54" s="87" t="inlineStr">
@@ -15913,7 +15913,7 @@
     <row r="57" ht="40.05" customHeight="1" s="82">
       <c r="A57" s="87" t="inlineStr">
         <is>
-          <t>P6-S25</t>
+          <t>P6-S33</t>
         </is>
       </c>
       <c r="B57" s="87" t="inlineStr">
@@ -15966,7 +15966,7 @@
       </c>
       <c r="N57" s="87" t="inlineStr">
         <is>
-          <t>P6-R02</t>
+          <t>P6-R26</t>
         </is>
       </c>
       <c r="O57" s="87" t="inlineStr">
@@ -15978,7 +15978,7 @@
     <row r="58" ht="40.05" customHeight="1" s="82">
       <c r="A58" s="87" t="inlineStr">
         <is>
-          <t>P6-S27</t>
+          <t>P6-S34</t>
         </is>
       </c>
       <c r="B58" s="87" t="inlineStr">
@@ -16059,7 +16059,7 @@
     <row r="63" ht="40.05" customHeight="1" s="82">
       <c r="A63" s="87" t="inlineStr">
         <is>
-          <t>P6-D01</t>
+          <t>P6-D35</t>
         </is>
       </c>
       <c r="B63" s="87" t="inlineStr">
@@ -16117,7 +16117,7 @@
       </c>
       <c r="N63" s="87" t="inlineStr">
         <is>
-          <t>P6-F06</t>
+          <t>P6-F15</t>
         </is>
       </c>
       <c r="O63" s="87" t="inlineStr">
@@ -16129,7 +16129,7 @@
     <row r="64" ht="40.05" customHeight="1" s="82">
       <c r="A64" s="87" t="inlineStr">
         <is>
-          <t>P6-D02</t>
+          <t>P6-D36</t>
         </is>
       </c>
       <c r="B64" s="87" t="inlineStr">
@@ -16187,7 +16187,7 @@
       </c>
       <c r="N64" s="87" t="inlineStr">
         <is>
-          <t>P6-D01</t>
+          <t>P6-D35</t>
         </is>
       </c>
       <c r="O64" s="87" t="inlineStr">
@@ -16199,7 +16199,7 @@
     <row r="65" ht="40.05" customHeight="1" s="82">
       <c r="A65" s="87" t="inlineStr">
         <is>
-          <t>P6-D03</t>
+          <t>P6-D37</t>
         </is>
       </c>
       <c r="B65" s="87" t="inlineStr">
@@ -16257,7 +16257,7 @@
       </c>
       <c r="N65" s="87" t="inlineStr">
         <is>
-          <t>P6-D02</t>
+          <t>P6-D36</t>
         </is>
       </c>
       <c r="O65" s="87" t="inlineStr">
@@ -16335,7 +16335,7 @@
       </c>
       <c r="N68" s="87" t="inlineStr">
         <is>
-          <t>P6-D03</t>
+          <t>P6-D37</t>
         </is>
       </c>
       <c r="O68" s="87" t="inlineStr">
@@ -16715,7 +16715,7 @@
       </c>
       <c r="C4" s="18" t="inlineStr">
         <is>
-          <t>P6-D01 — updated P6-S01/S02/S03</t>
+          <t>P6-D35 — updated P6-S01/S02/S03</t>
         </is>
       </c>
       <c r="D4" s="25" t="inlineStr">
@@ -16781,7 +16781,7 @@
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>P6-S16 — NEW</t>
+          <t>P6-S31 — NEW</t>
         </is>
       </c>
       <c r="D7" s="25" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>P6-S01, P6-S10, P6-S13, P6-S16</t>
+          <t>P6-S01, P6-S10, P6-S13, P6-S31</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
@@ -16869,7 +16869,7 @@
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>P6-S02, P6-S13, P6-S16</t>
+          <t>P6-S02, P6-S13, P6-S31</t>
         </is>
       </c>
       <c r="D11" s="26" t="inlineStr">
@@ -16891,7 +16891,7 @@
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>P6-S01, P6-S03, P6-S13, P6-S16</t>
+          <t>P6-S01, P6-S03, P6-S13, P6-S31</t>
         </is>
       </c>
       <c r="D12" s="26" t="inlineStr">
@@ -16913,7 +16913,7 @@
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>P6-S01, P6-D03</t>
+          <t>P6-S01, P6-D37</t>
         </is>
       </c>
       <c r="D13" s="26" t="inlineStr">
@@ -16957,7 +16957,7 @@
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>P6-D03</t>
+          <t>P6-D37</t>
         </is>
       </c>
       <c r="D15" s="26" t="inlineStr">

</xml_diff>